<commit_message>
Update the lexicon files
</commit_message>
<xml_diff>
--- a/data/lexicon_review/Lebanese.xlsx
+++ b/data/lexicon_review/Lebanese.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1155,17 +1155,17 @@
           <t>ي</t>
         </is>
       </c>
-      <c r="F20" t="inlineStr"/>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>ا</t>
+        </is>
+      </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>ا</t>
-        </is>
-      </c>
-      <c r="H20" t="inlineStr">
-        <is>
           <t>م</t>
         </is>
       </c>
+      <c r="H20" t="inlineStr"/>
       <c r="I20" t="inlineStr"/>
       <c r="J20" t="inlineStr"/>
       <c r="K20" t="inlineStr"/>
@@ -1181,32 +1181,32 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>ayam</t>
+          <t>iyam</t>
         </is>
       </c>
       <c r="B21" t="inlineStr"/>
       <c r="C21" t="inlineStr"/>
-      <c r="D21" t="inlineStr"/>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>i</t>
+        </is>
+      </c>
       <c r="E21" t="inlineStr">
         <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
           <t>a</t>
         </is>
       </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>y</t>
-        </is>
-      </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>a</t>
-        </is>
-      </c>
-      <c r="H21" t="inlineStr">
-        <is>
           <t>m</t>
         </is>
       </c>
+      <c r="H21" t="inlineStr"/>
       <c r="I21" t="inlineStr"/>
       <c r="J21" t="inlineStr"/>
       <c r="K21" t="inlineStr"/>
@@ -1247,7 +1247,7 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C23" t="inlineStr"/>
       <c r="D23" t="inlineStr">
@@ -1260,17 +1260,17 @@
           <t>ي</t>
         </is>
       </c>
-      <c r="F23" t="inlineStr">
+      <c r="F23" t="inlineStr"/>
+      <c r="G23" t="inlineStr">
         <is>
           <t>ا</t>
         </is>
       </c>
-      <c r="G23" t="inlineStr">
+      <c r="H23" t="inlineStr">
         <is>
           <t>م</t>
         </is>
       </c>
-      <c r="H23" t="inlineStr"/>
       <c r="I23" t="inlineStr"/>
       <c r="J23" t="inlineStr"/>
       <c r="K23" t="inlineStr"/>
@@ -1286,32 +1286,32 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>iyem</t>
+          <t>ayam</t>
         </is>
       </c>
       <c r="B24" t="inlineStr"/>
       <c r="C24" t="inlineStr"/>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>i</t>
-        </is>
-      </c>
+      <c r="D24" t="inlineStr"/>
       <c r="E24" t="inlineStr">
         <is>
+          <t>a</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
           <t>y</t>
         </is>
       </c>
-      <c r="F24" t="inlineStr">
-        <is>
-          <t>e</t>
-        </is>
-      </c>
       <c r="G24" t="inlineStr">
         <is>
+          <t>a</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
           <t>m</t>
         </is>
       </c>
-      <c r="H24" t="inlineStr"/>
       <c r="I24" t="inlineStr"/>
       <c r="J24" t="inlineStr"/>
       <c r="K24" t="inlineStr"/>
@@ -1352,7 +1352,7 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C26" t="inlineStr"/>
       <c r="D26" t="inlineStr">
@@ -1391,7 +1391,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>iyam</t>
+          <t>iyem</t>
         </is>
       </c>
       <c r="B27" t="inlineStr"/>
@@ -1408,7 +1408,7 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>a</t>
+          <t>e</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -1457,7 +1457,7 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="C29" t="inlineStr"/>
       <c r="D29" t="inlineStr">
@@ -1470,17 +1470,17 @@
           <t>ي</t>
         </is>
       </c>
-      <c r="F29" t="inlineStr"/>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>ا</t>
+        </is>
+      </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>ا</t>
-        </is>
-      </c>
-      <c r="H29" t="inlineStr">
-        <is>
           <t>م</t>
         </is>
       </c>
+      <c r="H29" t="inlineStr"/>
       <c r="I29" t="inlineStr"/>
       <c r="J29" t="inlineStr"/>
       <c r="K29" t="inlineStr"/>
@@ -1496,36 +1496,32 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2eyem</t>
+          <t>iyyem</t>
         </is>
       </c>
       <c r="B30" t="inlineStr"/>
       <c r="C30" t="inlineStr"/>
       <c r="D30" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>i</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
+          <t>yy</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
           <t>e</t>
         </is>
       </c>
-      <c r="F30" t="inlineStr">
-        <is>
-          <t>y</t>
-        </is>
-      </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>e</t>
-        </is>
-      </c>
-      <c r="H30" t="inlineStr">
-        <is>
           <t>m</t>
         </is>
       </c>
+      <c r="H30" t="inlineStr"/>
       <c r="I30" t="inlineStr"/>
       <c r="J30" t="inlineStr"/>
       <c r="K30" t="inlineStr"/>
@@ -1579,17 +1575,17 @@
           <t>ي</t>
         </is>
       </c>
-      <c r="F32" t="inlineStr">
+      <c r="F32" t="inlineStr"/>
+      <c r="G32" t="inlineStr">
         <is>
           <t>ا</t>
         </is>
       </c>
-      <c r="G32" t="inlineStr">
+      <c r="H32" t="inlineStr">
         <is>
           <t>م</t>
         </is>
       </c>
-      <c r="H32" t="inlineStr"/>
       <c r="I32" t="inlineStr"/>
       <c r="J32" t="inlineStr"/>
       <c r="K32" t="inlineStr"/>
@@ -1605,32 +1601,36 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>eyyem</t>
+          <t>2iyem</t>
         </is>
       </c>
       <c r="B33" t="inlineStr"/>
       <c r="C33" t="inlineStr"/>
       <c r="D33" t="inlineStr">
         <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>i</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
           <t>e</t>
         </is>
       </c>
-      <c r="E33" t="inlineStr">
-        <is>
-          <t>yy</t>
-        </is>
-      </c>
-      <c r="F33" t="inlineStr">
-        <is>
-          <t>e</t>
-        </is>
-      </c>
-      <c r="G33" t="inlineStr">
+      <c r="H33" t="inlineStr">
         <is>
           <t>m</t>
         </is>
       </c>
-      <c r="H33" t="inlineStr"/>
       <c r="I33" t="inlineStr"/>
       <c r="J33" t="inlineStr"/>
       <c r="K33" t="inlineStr"/>
@@ -1710,7 +1710,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2iyem</t>
+          <t>2eyem</t>
         </is>
       </c>
       <c r="B36" t="inlineStr"/>
@@ -1722,7 +1722,7 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>i</t>
+          <t>e</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
@@ -1780,7 +1780,7 @@
         </is>
       </c>
       <c r="B38" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="C38" t="inlineStr"/>
       <c r="D38" t="inlineStr">
@@ -1819,14 +1819,14 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>iyyem</t>
+          <t>eyyem</t>
         </is>
       </c>
       <c r="B39" t="inlineStr"/>
       <c r="C39" t="inlineStr"/>
       <c r="D39" t="inlineStr">
         <is>
-          <t>i</t>
+          <t>e</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
@@ -2196,7 +2196,7 @@
         </is>
       </c>
       <c r="B50" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C50" t="inlineStr"/>
       <c r="D50" t="inlineStr">
@@ -2204,18 +2204,18 @@
           <t>آ</t>
         </is>
       </c>
-      <c r="E50" t="inlineStr">
+      <c r="E50" t="inlineStr"/>
+      <c r="F50" t="inlineStr">
         <is>
           <t>خ</t>
         </is>
       </c>
-      <c r="F50" t="inlineStr"/>
-      <c r="G50" t="inlineStr">
+      <c r="G50" t="inlineStr"/>
+      <c r="H50" t="inlineStr">
         <is>
           <t>ر</t>
         </is>
       </c>
-      <c r="H50" t="inlineStr"/>
       <c r="I50" t="inlineStr"/>
       <c r="J50" t="inlineStr"/>
       <c r="K50" t="inlineStr"/>
@@ -2231,32 +2231,36 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>ekhir</t>
+          <t>2e5er</t>
         </is>
       </c>
       <c r="B51" t="inlineStr"/>
       <c r="C51" t="inlineStr"/>
       <c r="D51" t="inlineStr">
         <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
           <t>e</t>
         </is>
       </c>
-      <c r="E51" t="inlineStr">
-        <is>
-          <t>kh</t>
-        </is>
-      </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>i</t>
+          <t>5</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
         <is>
+          <t>e</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
           <t>r</t>
         </is>
       </c>
-      <c r="H51" t="inlineStr"/>
       <c r="I51" t="inlineStr"/>
       <c r="J51" t="inlineStr"/>
       <c r="K51" t="inlineStr"/>
@@ -2305,18 +2309,18 @@
           <t>آ</t>
         </is>
       </c>
-      <c r="E53" t="inlineStr">
+      <c r="E53" t="inlineStr"/>
+      <c r="F53" t="inlineStr">
         <is>
           <t>خ</t>
         </is>
       </c>
-      <c r="F53" t="inlineStr"/>
-      <c r="G53" t="inlineStr">
+      <c r="G53" t="inlineStr"/>
+      <c r="H53" t="inlineStr">
         <is>
           <t>ر</t>
         </is>
       </c>
-      <c r="H53" t="inlineStr"/>
       <c r="I53" t="inlineStr"/>
       <c r="J53" t="inlineStr"/>
       <c r="K53" t="inlineStr"/>
@@ -2332,32 +2336,36 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>akhar</t>
+          <t>2a5ar</t>
         </is>
       </c>
       <c r="B54" t="inlineStr"/>
       <c r="C54" t="inlineStr"/>
       <c r="D54" t="inlineStr">
         <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
           <t>a</t>
         </is>
       </c>
-      <c r="E54" t="inlineStr">
-        <is>
-          <t>kh</t>
-        </is>
-      </c>
       <c r="F54" t="inlineStr">
         <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
           <t>a</t>
         </is>
       </c>
-      <c r="G54" t="inlineStr">
+      <c r="H54" t="inlineStr">
         <is>
           <t>r</t>
         </is>
       </c>
-      <c r="H54" t="inlineStr"/>
       <c r="I54" t="inlineStr"/>
       <c r="J54" t="inlineStr"/>
       <c r="K54" t="inlineStr"/>
@@ -2433,7 +2441,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>ekher</t>
+          <t>ekhir</t>
         </is>
       </c>
       <c r="B57" t="inlineStr"/>
@@ -2450,7 +2458,7 @@
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>e</t>
+          <t>i</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
@@ -2499,7 +2507,7 @@
         </is>
       </c>
       <c r="B59" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C59" t="inlineStr"/>
       <c r="D59" t="inlineStr">
@@ -2507,18 +2515,18 @@
           <t>آ</t>
         </is>
       </c>
-      <c r="E59" t="inlineStr"/>
-      <c r="F59" t="inlineStr">
+      <c r="E59" t="inlineStr">
         <is>
           <t>خ</t>
         </is>
       </c>
-      <c r="G59" t="inlineStr"/>
-      <c r="H59" t="inlineStr">
+      <c r="F59" t="inlineStr"/>
+      <c r="G59" t="inlineStr">
         <is>
           <t>ر</t>
         </is>
       </c>
+      <c r="H59" t="inlineStr"/>
       <c r="I59" t="inlineStr"/>
       <c r="J59" t="inlineStr"/>
       <c r="K59" t="inlineStr"/>
@@ -2534,36 +2542,32 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>2a5ar</t>
+          <t>ekher</t>
         </is>
       </c>
       <c r="B60" t="inlineStr"/>
       <c r="C60" t="inlineStr"/>
       <c r="D60" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>e</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>a</t>
+          <t>kh</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>e</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>a</t>
-        </is>
-      </c>
-      <c r="H60" t="inlineStr">
-        <is>
           <t>r</t>
         </is>
       </c>
+      <c r="H60" t="inlineStr"/>
       <c r="I60" t="inlineStr"/>
       <c r="J60" t="inlineStr"/>
       <c r="K60" t="inlineStr"/>
@@ -2612,18 +2616,18 @@
           <t>آ</t>
         </is>
       </c>
-      <c r="E62" t="inlineStr"/>
-      <c r="F62" t="inlineStr">
+      <c r="E62" t="inlineStr">
         <is>
           <t>خ</t>
         </is>
       </c>
-      <c r="G62" t="inlineStr"/>
-      <c r="H62" t="inlineStr">
+      <c r="F62" t="inlineStr"/>
+      <c r="G62" t="inlineStr">
         <is>
           <t>ر</t>
         </is>
       </c>
+      <c r="H62" t="inlineStr"/>
       <c r="I62" t="inlineStr"/>
       <c r="J62" t="inlineStr"/>
       <c r="K62" t="inlineStr"/>
@@ -2639,36 +2643,32 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2e5er</t>
+          <t>akhar</t>
         </is>
       </c>
       <c r="B63" t="inlineStr"/>
       <c r="C63" t="inlineStr"/>
       <c r="D63" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>a</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>e</t>
+          <t>kh</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>a</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>e</t>
-        </is>
-      </c>
-      <c r="H63" t="inlineStr">
-        <is>
           <t>r</t>
         </is>
       </c>
+      <c r="H63" t="inlineStr"/>
       <c r="I63" t="inlineStr"/>
       <c r="J63" t="inlineStr"/>
       <c r="K63" t="inlineStr"/>
@@ -3210,7 +3210,7 @@
         </is>
       </c>
       <c r="B80" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C80" t="inlineStr"/>
       <c r="D80" t="inlineStr">
@@ -3218,22 +3218,22 @@
           <t>ر</t>
         </is>
       </c>
-      <c r="E80" t="inlineStr"/>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>ئ</t>
+        </is>
+      </c>
       <c r="F80" t="inlineStr">
         <is>
-          <t>ئ</t>
+          <t>ي</t>
         </is>
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>ي</t>
-        </is>
-      </c>
-      <c r="H80" t="inlineStr">
-        <is>
           <t>س</t>
         </is>
       </c>
+      <c r="H80" t="inlineStr"/>
       <c r="I80" t="inlineStr"/>
       <c r="J80" t="inlineStr"/>
       <c r="K80" t="inlineStr"/>
@@ -3249,7 +3249,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>ra2iss</t>
+          <t>raeiss</t>
         </is>
       </c>
       <c r="B81" t="inlineStr"/>
@@ -3266,19 +3266,15 @@
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>ei</t>
         </is>
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>i</t>
-        </is>
-      </c>
-      <c r="H81" t="inlineStr">
-        <is>
           <t>ss</t>
         </is>
       </c>
+      <c r="H81" t="inlineStr"/>
       <c r="I81" t="inlineStr"/>
       <c r="J81" t="inlineStr"/>
       <c r="K81" t="inlineStr"/>
@@ -3319,7 +3315,7 @@
         </is>
       </c>
       <c r="B83" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C83" t="inlineStr"/>
       <c r="D83" t="inlineStr">
@@ -3327,22 +3323,22 @@
           <t>ر</t>
         </is>
       </c>
-      <c r="E83" t="inlineStr">
+      <c r="E83" t="inlineStr"/>
+      <c r="F83" t="inlineStr">
         <is>
           <t>ئ</t>
         </is>
       </c>
-      <c r="F83" t="inlineStr">
+      <c r="G83" t="inlineStr">
         <is>
           <t>ي</t>
         </is>
       </c>
-      <c r="G83" t="inlineStr">
+      <c r="H83" t="inlineStr">
         <is>
           <t>س</t>
         </is>
       </c>
-      <c r="H83" t="inlineStr"/>
       <c r="I83" t="inlineStr"/>
       <c r="J83" t="inlineStr"/>
       <c r="K83" t="inlineStr"/>
@@ -3358,7 +3354,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>raeiss</t>
+          <t>ra2iss</t>
         </is>
       </c>
       <c r="B84" t="inlineStr"/>
@@ -3375,15 +3371,19 @@
       </c>
       <c r="F84" t="inlineStr">
         <is>
-          <t>ei</t>
+          <t>2</t>
         </is>
       </c>
       <c r="G84" t="inlineStr">
         <is>
+          <t>i</t>
+        </is>
+      </c>
+      <c r="H84" t="inlineStr">
+        <is>
           <t>ss</t>
         </is>
       </c>
-      <c r="H84" t="inlineStr"/>
       <c r="I84" t="inlineStr"/>
       <c r="J84" t="inlineStr"/>
       <c r="K84" t="inlineStr"/>
@@ -3642,30 +3642,14 @@
         </is>
       </c>
       <c r="B92" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C92" t="inlineStr"/>
-      <c r="D92" t="inlineStr">
-        <is>
-          <t>س</t>
-        </is>
-      </c>
-      <c r="E92" t="inlineStr">
-        <is>
-          <t>ؤ</t>
-        </is>
-      </c>
-      <c r="F92" t="inlineStr">
-        <is>
-          <t>ا</t>
-        </is>
-      </c>
+      <c r="D92" t="inlineStr"/>
+      <c r="E92" t="inlineStr"/>
+      <c r="F92" t="inlineStr"/>
       <c r="G92" t="inlineStr"/>
-      <c r="H92" t="inlineStr">
-        <is>
-          <t>ل</t>
-        </is>
-      </c>
+      <c r="H92" t="inlineStr"/>
       <c r="I92" t="inlineStr"/>
       <c r="J92" t="inlineStr"/>
       <c r="K92" t="inlineStr"/>
@@ -3681,36 +3665,16 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>sou2al</t>
+          <t>sou’al</t>
         </is>
       </c>
       <c r="B93" t="inlineStr"/>
       <c r="C93" t="inlineStr"/>
-      <c r="D93" t="inlineStr">
-        <is>
-          <t>s</t>
-        </is>
-      </c>
-      <c r="E93" t="inlineStr">
-        <is>
-          <t>ou</t>
-        </is>
-      </c>
-      <c r="F93" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="G93" t="inlineStr">
-        <is>
-          <t>a</t>
-        </is>
-      </c>
-      <c r="H93" t="inlineStr">
-        <is>
-          <t>l</t>
-        </is>
-      </c>
+      <c r="D93" t="inlineStr"/>
+      <c r="E93" t="inlineStr"/>
+      <c r="F93" t="inlineStr"/>
+      <c r="G93" t="inlineStr"/>
+      <c r="H93" t="inlineStr"/>
       <c r="I93" t="inlineStr"/>
       <c r="J93" t="inlineStr"/>
       <c r="K93" t="inlineStr"/>
@@ -3751,14 +3715,30 @@
         </is>
       </c>
       <c r="B95" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="C95" t="inlineStr"/>
-      <c r="D95" t="inlineStr"/>
-      <c r="E95" t="inlineStr"/>
-      <c r="F95" t="inlineStr"/>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>س</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>ؤ</t>
+        </is>
+      </c>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>ا</t>
+        </is>
+      </c>
       <c r="G95" t="inlineStr"/>
-      <c r="H95" t="inlineStr"/>
+      <c r="H95" t="inlineStr">
+        <is>
+          <t>ل</t>
+        </is>
+      </c>
       <c r="I95" t="inlineStr"/>
       <c r="J95" t="inlineStr"/>
       <c r="K95" t="inlineStr"/>
@@ -3774,16 +3754,36 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>sou’al</t>
+          <t>sou2el</t>
         </is>
       </c>
       <c r="B96" t="inlineStr"/>
       <c r="C96" t="inlineStr"/>
-      <c r="D96" t="inlineStr"/>
-      <c r="E96" t="inlineStr"/>
-      <c r="F96" t="inlineStr"/>
-      <c r="G96" t="inlineStr"/>
-      <c r="H96" t="inlineStr"/>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>s</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>ou</t>
+        </is>
+      </c>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="G96" t="inlineStr">
+        <is>
+          <t>e</t>
+        </is>
+      </c>
+      <c r="H96" t="inlineStr">
+        <is>
+          <t>l</t>
+        </is>
+      </c>
       <c r="I96" t="inlineStr"/>
       <c r="J96" t="inlineStr"/>
       <c r="K96" t="inlineStr"/>
@@ -3824,7 +3824,7 @@
         </is>
       </c>
       <c r="B98" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="C98" t="inlineStr"/>
       <c r="D98" t="inlineStr">
@@ -3863,7 +3863,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>sou2el</t>
+          <t>sou2al</t>
         </is>
       </c>
       <c r="B99" t="inlineStr"/>
@@ -3885,7 +3885,7 @@
       </c>
       <c r="G99" t="inlineStr">
         <is>
-          <t>e</t>
+          <t>a</t>
         </is>
       </c>
       <c r="H99" t="inlineStr">
@@ -3933,7 +3933,7 @@
         </is>
       </c>
       <c r="B101" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="C101" t="inlineStr"/>
       <c r="D101" t="inlineStr">
@@ -3951,12 +3951,12 @@
           <t>ت</t>
         </is>
       </c>
-      <c r="G101" t="inlineStr">
+      <c r="G101" t="inlineStr"/>
+      <c r="H101" t="inlineStr">
         <is>
           <t>ع</t>
         </is>
       </c>
-      <c r="H101" t="inlineStr"/>
       <c r="I101" t="inlineStr">
         <is>
           <t>م</t>
@@ -3984,7 +3984,7 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>esteemel</t>
+          <t>este3mel</t>
         </is>
       </c>
       <c r="B102" t="inlineStr"/>
@@ -4011,7 +4011,7 @@
       </c>
       <c r="H102" t="inlineStr">
         <is>
-          <t>e</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I102" t="inlineStr">
@@ -4066,7 +4066,7 @@
         </is>
       </c>
       <c r="B104" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="C104" t="inlineStr"/>
       <c r="D104" t="inlineStr">
@@ -4117,31 +4117,31 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>este3mel</t>
+          <t>iste3mal</t>
         </is>
       </c>
       <c r="B105" t="inlineStr"/>
       <c r="C105" t="inlineStr"/>
       <c r="D105" t="inlineStr">
         <is>
+          <t>i</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>s</t>
+        </is>
+      </c>
+      <c r="F105" t="inlineStr">
+        <is>
+          <t>t</t>
+        </is>
+      </c>
+      <c r="G105" t="inlineStr">
+        <is>
           <t>e</t>
         </is>
       </c>
-      <c r="E105" t="inlineStr">
-        <is>
-          <t>s</t>
-        </is>
-      </c>
-      <c r="F105" t="inlineStr">
-        <is>
-          <t>t</t>
-        </is>
-      </c>
-      <c r="G105" t="inlineStr">
-        <is>
-          <t>e</t>
-        </is>
-      </c>
       <c r="H105" t="inlineStr">
         <is>
           <t>3</t>
@@ -4154,7 +4154,7 @@
       </c>
       <c r="J105" t="inlineStr">
         <is>
-          <t>e</t>
+          <t>a</t>
         </is>
       </c>
       <c r="K105" t="inlineStr">
@@ -4250,7 +4250,7 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>isti3mal</t>
+          <t>iste3mel</t>
         </is>
       </c>
       <c r="B108" t="inlineStr"/>
@@ -4272,7 +4272,7 @@
       </c>
       <c r="G108" t="inlineStr">
         <is>
-          <t>i</t>
+          <t>e</t>
         </is>
       </c>
       <c r="H108" t="inlineStr">
@@ -4287,7 +4287,7 @@
       </c>
       <c r="J108" t="inlineStr">
         <is>
-          <t>a</t>
+          <t>e</t>
         </is>
       </c>
       <c r="K108" t="inlineStr">
@@ -4350,12 +4350,12 @@
           <t>ت</t>
         </is>
       </c>
-      <c r="G110" t="inlineStr"/>
-      <c r="H110" t="inlineStr">
+      <c r="G110" t="inlineStr">
         <is>
           <t>ع</t>
         </is>
       </c>
+      <c r="H110" t="inlineStr"/>
       <c r="I110" t="inlineStr">
         <is>
           <t>م</t>
@@ -4383,14 +4383,14 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>iste3mal</t>
+          <t>esteemel</t>
         </is>
       </c>
       <c r="B111" t="inlineStr"/>
       <c r="C111" t="inlineStr"/>
       <c r="D111" t="inlineStr">
         <is>
-          <t>i</t>
+          <t>e</t>
         </is>
       </c>
       <c r="E111" t="inlineStr">
@@ -4410,7 +4410,7 @@
       </c>
       <c r="H111" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>e</t>
         </is>
       </c>
       <c r="I111" t="inlineStr">
@@ -4420,7 +4420,7 @@
       </c>
       <c r="J111" t="inlineStr">
         <is>
-          <t>a</t>
+          <t>e</t>
         </is>
       </c>
       <c r="K111" t="inlineStr">
@@ -4516,7 +4516,7 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>iste3mel</t>
+          <t>isti3mal</t>
         </is>
       </c>
       <c r="B114" t="inlineStr"/>
@@ -4538,7 +4538,7 @@
       </c>
       <c r="G114" t="inlineStr">
         <is>
-          <t>e</t>
+          <t>i</t>
         </is>
       </c>
       <c r="H114" t="inlineStr">
@@ -4553,7 +4553,7 @@
       </c>
       <c r="J114" t="inlineStr">
         <is>
-          <t>e</t>
+          <t>a</t>
         </is>
       </c>
       <c r="K114" t="inlineStr">
@@ -4735,7 +4735,7 @@
         </is>
       </c>
       <c r="B119" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="C119" t="inlineStr"/>
       <c r="D119" t="inlineStr">
@@ -4774,7 +4774,7 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>salem</t>
+          <t>salam</t>
         </is>
       </c>
       <c r="B120" t="inlineStr"/>
@@ -4796,7 +4796,7 @@
       </c>
       <c r="G120" t="inlineStr">
         <is>
-          <t>e</t>
+          <t>a</t>
         </is>
       </c>
       <c r="H120" t="inlineStr">
@@ -4844,7 +4844,7 @@
         </is>
       </c>
       <c r="B122" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="C122" t="inlineStr"/>
       <c r="D122" t="inlineStr">
@@ -4883,7 +4883,7 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>salam</t>
+          <t>salem</t>
         </is>
       </c>
       <c r="B123" t="inlineStr"/>
@@ -4905,7 +4905,7 @@
       </c>
       <c r="G123" t="inlineStr">
         <is>
-          <t>a</t>
+          <t>e</t>
         </is>
       </c>
       <c r="H123" t="inlineStr">
@@ -4953,7 +4953,7 @@
         </is>
       </c>
       <c r="B125" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C125" t="inlineStr"/>
       <c r="D125" t="inlineStr">
@@ -4971,18 +4971,18 @@
           <t>ت</t>
         </is>
       </c>
-      <c r="G125" t="inlineStr"/>
-      <c r="H125" t="inlineStr">
+      <c r="G125" t="inlineStr">
         <is>
           <t>ع</t>
         </is>
       </c>
-      <c r="I125" t="inlineStr"/>
-      <c r="J125" t="inlineStr">
+      <c r="H125" t="inlineStr"/>
+      <c r="I125" t="inlineStr">
         <is>
           <t>م</t>
         </is>
       </c>
+      <c r="J125" t="inlineStr"/>
       <c r="K125" t="inlineStr">
         <is>
           <t>ل</t>
@@ -5008,7 +5008,7 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>sta3emlo</t>
+          <t>staamalo</t>
         </is>
       </c>
       <c r="B126" t="inlineStr"/>
@@ -5031,17 +5031,17 @@
       </c>
       <c r="H126" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>a</t>
         </is>
       </c>
       <c r="I126" t="inlineStr">
         <is>
-          <t>e</t>
+          <t>m</t>
         </is>
       </c>
       <c r="J126" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>a</t>
         </is>
       </c>
       <c r="K126" t="inlineStr">
@@ -5090,7 +5090,7 @@
         </is>
       </c>
       <c r="B128" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C128" t="inlineStr"/>
       <c r="D128" t="inlineStr">
@@ -5108,12 +5108,12 @@
           <t>ت</t>
         </is>
       </c>
-      <c r="G128" t="inlineStr">
+      <c r="G128" t="inlineStr"/>
+      <c r="H128" t="inlineStr">
         <is>
           <t>ع</t>
         </is>
       </c>
-      <c r="H128" t="inlineStr"/>
       <c r="I128" t="inlineStr">
         <is>
           <t>م</t>
@@ -5145,7 +5145,7 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>staamalo</t>
+          <t>sta3malo</t>
         </is>
       </c>
       <c r="B129" t="inlineStr"/>
@@ -5168,7 +5168,7 @@
       </c>
       <c r="H129" t="inlineStr">
         <is>
-          <t>a</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I129" t="inlineStr">
@@ -5227,7 +5227,7 @@
         </is>
       </c>
       <c r="B131" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C131" t="inlineStr"/>
       <c r="D131" t="inlineStr">
@@ -5251,12 +5251,12 @@
           <t>ع</t>
         </is>
       </c>
-      <c r="I131" t="inlineStr">
+      <c r="I131" t="inlineStr"/>
+      <c r="J131" t="inlineStr">
         <is>
           <t>م</t>
         </is>
       </c>
-      <c r="J131" t="inlineStr"/>
       <c r="K131" t="inlineStr">
         <is>
           <t>ل</t>
@@ -5282,7 +5282,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>sta3malo</t>
+          <t>sta3emlo</t>
         </is>
       </c>
       <c r="B132" t="inlineStr"/>
@@ -5310,12 +5310,12 @@
       </c>
       <c r="I132" t="inlineStr">
         <is>
+          <t>e</t>
+        </is>
+      </c>
+      <c r="J132" t="inlineStr">
+        <is>
           <t>m</t>
-        </is>
-      </c>
-      <c r="J132" t="inlineStr">
-        <is>
-          <t>a</t>
         </is>
       </c>
       <c r="K132" t="inlineStr">
@@ -5382,18 +5382,18 @@
           <t>ت</t>
         </is>
       </c>
-      <c r="G134" t="inlineStr"/>
-      <c r="H134" t="inlineStr">
+      <c r="G134" t="inlineStr">
         <is>
           <t>ع</t>
         </is>
       </c>
-      <c r="I134" t="inlineStr"/>
-      <c r="J134" t="inlineStr">
+      <c r="H134" t="inlineStr"/>
+      <c r="I134" t="inlineStr">
         <is>
           <t>م</t>
         </is>
       </c>
+      <c r="J134" t="inlineStr"/>
       <c r="K134" t="inlineStr">
         <is>
           <t>ل</t>
@@ -5419,7 +5419,7 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>esta3emlo</t>
+          <t>estaamalo</t>
         </is>
       </c>
       <c r="B135" t="inlineStr"/>
@@ -5446,17 +5446,17 @@
       </c>
       <c r="H135" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>a</t>
         </is>
       </c>
       <c r="I135" t="inlineStr">
         <is>
-          <t>e</t>
+          <t>m</t>
         </is>
       </c>
       <c r="J135" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>a</t>
         </is>
       </c>
       <c r="K135" t="inlineStr">
@@ -5523,12 +5523,12 @@
           <t>ت</t>
         </is>
       </c>
-      <c r="G137" t="inlineStr">
+      <c r="G137" t="inlineStr"/>
+      <c r="H137" t="inlineStr">
         <is>
           <t>ع</t>
         </is>
       </c>
-      <c r="H137" t="inlineStr"/>
       <c r="I137" t="inlineStr">
         <is>
           <t>م</t>
@@ -5560,44 +5560,44 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>estaamalo</t>
+          <t>ista3melo</t>
         </is>
       </c>
       <c r="B138" t="inlineStr"/>
       <c r="C138" t="inlineStr"/>
       <c r="D138" t="inlineStr">
         <is>
+          <t>i</t>
+        </is>
+      </c>
+      <c r="E138" t="inlineStr">
+        <is>
+          <t>s</t>
+        </is>
+      </c>
+      <c r="F138" t="inlineStr">
+        <is>
+          <t>t</t>
+        </is>
+      </c>
+      <c r="G138" t="inlineStr">
+        <is>
+          <t>a</t>
+        </is>
+      </c>
+      <c r="H138" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="I138" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="J138" t="inlineStr">
+        <is>
           <t>e</t>
-        </is>
-      </c>
-      <c r="E138" t="inlineStr">
-        <is>
-          <t>s</t>
-        </is>
-      </c>
-      <c r="F138" t="inlineStr">
-        <is>
-          <t>t</t>
-        </is>
-      </c>
-      <c r="G138" t="inlineStr">
-        <is>
-          <t>a</t>
-        </is>
-      </c>
-      <c r="H138" t="inlineStr">
-        <is>
-          <t>a</t>
-        </is>
-      </c>
-      <c r="I138" t="inlineStr">
-        <is>
-          <t>m</t>
-        </is>
-      </c>
-      <c r="J138" t="inlineStr">
-        <is>
-          <t>a</t>
         </is>
       </c>
       <c r="K138" t="inlineStr">
@@ -5646,7 +5646,7 @@
         </is>
       </c>
       <c r="B140" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C140" t="inlineStr"/>
       <c r="D140" t="inlineStr">
@@ -5701,16 +5701,12 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>ista3melo</t>
+          <t>sta3malou</t>
         </is>
       </c>
       <c r="B141" t="inlineStr"/>
       <c r="C141" t="inlineStr"/>
-      <c r="D141" t="inlineStr">
-        <is>
-          <t>i</t>
-        </is>
-      </c>
+      <c r="D141" t="inlineStr"/>
       <c r="E141" t="inlineStr">
         <is>
           <t>s</t>
@@ -5738,7 +5734,7 @@
       </c>
       <c r="J141" t="inlineStr">
         <is>
-          <t>e</t>
+          <t>a</t>
         </is>
       </c>
       <c r="K141" t="inlineStr">
@@ -5748,7 +5744,7 @@
       </c>
       <c r="L141" t="inlineStr">
         <is>
-          <t>o</t>
+          <t>ou</t>
         </is>
       </c>
       <c r="M141" t="inlineStr"/>
@@ -5787,7 +5783,7 @@
         </is>
       </c>
       <c r="B143" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C143" t="inlineStr"/>
       <c r="D143" t="inlineStr">
@@ -5811,12 +5807,12 @@
           <t>ع</t>
         </is>
       </c>
-      <c r="I143" t="inlineStr">
+      <c r="I143" t="inlineStr"/>
+      <c r="J143" t="inlineStr">
         <is>
           <t>م</t>
         </is>
       </c>
-      <c r="J143" t="inlineStr"/>
       <c r="K143" t="inlineStr">
         <is>
           <t>ل</t>
@@ -5842,12 +5838,16 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>sta3malou</t>
+          <t>esta3emlo</t>
         </is>
       </c>
       <c r="B144" t="inlineStr"/>
       <c r="C144" t="inlineStr"/>
-      <c r="D144" t="inlineStr"/>
+      <c r="D144" t="inlineStr">
+        <is>
+          <t>e</t>
+        </is>
+      </c>
       <c r="E144" t="inlineStr">
         <is>
           <t>s</t>
@@ -5870,14 +5870,14 @@
       </c>
       <c r="I144" t="inlineStr">
         <is>
+          <t>e</t>
+        </is>
+      </c>
+      <c r="J144" t="inlineStr">
+        <is>
           <t>m</t>
         </is>
       </c>
-      <c r="J144" t="inlineStr">
-        <is>
-          <t>a</t>
-        </is>
-      </c>
       <c r="K144" t="inlineStr">
         <is>
           <t>l</t>
@@ -5885,7 +5885,7 @@
       </c>
       <c r="L144" t="inlineStr">
         <is>
-          <t>ou</t>
+          <t>o</t>
         </is>
       </c>
       <c r="M144" t="inlineStr"/>
@@ -6569,7 +6569,7 @@
         </is>
       </c>
       <c r="B161" t="n">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="C161" t="inlineStr"/>
       <c r="D161" t="inlineStr">
@@ -6604,7 +6604,7 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>bab</t>
+          <t>beb</t>
         </is>
       </c>
       <c r="B162" t="inlineStr"/>
@@ -6616,7 +6616,7 @@
       </c>
       <c r="E162" t="inlineStr">
         <is>
-          <t>a</t>
+          <t>e</t>
         </is>
       </c>
       <c r="F162" t="inlineStr">
@@ -6666,7 +6666,7 @@
         </is>
       </c>
       <c r="B164" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="C164" t="inlineStr"/>
       <c r="D164" t="inlineStr">
@@ -6701,7 +6701,7 @@
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>beb</t>
+          <t>bab</t>
         </is>
       </c>
       <c r="B165" t="inlineStr"/>
@@ -6713,7 +6713,7 @@
       </c>
       <c r="E165" t="inlineStr">
         <is>
-          <t>e</t>
+          <t>a</t>
         </is>
       </c>
       <c r="F165" t="inlineStr">
@@ -6980,7 +6980,7 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>sawani</t>
+          <t>saweni</t>
         </is>
       </c>
       <c r="B174" t="inlineStr"/>
@@ -7002,7 +7002,7 @@
       </c>
       <c r="G174" t="inlineStr">
         <is>
-          <t>a</t>
+          <t>e</t>
         </is>
       </c>
       <c r="H174" t="inlineStr">
@@ -7214,7 +7214,7 @@
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>saweni</t>
+          <t>sawani</t>
         </is>
       </c>
       <c r="B180" t="inlineStr"/>
@@ -7236,7 +7236,7 @@
       </c>
       <c r="G180" t="inlineStr">
         <is>
-          <t>e</t>
+          <t>a</t>
         </is>
       </c>
       <c r="H180" t="inlineStr">
@@ -7797,7 +7797,7 @@
         </is>
       </c>
       <c r="B197" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="C197" t="inlineStr"/>
       <c r="D197" t="inlineStr">
@@ -7836,7 +7836,7 @@
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>djej</t>
+          <t>djaj</t>
         </is>
       </c>
       <c r="B198" t="inlineStr"/>
@@ -7853,7 +7853,7 @@
       </c>
       <c r="F198" t="inlineStr">
         <is>
-          <t>e</t>
+          <t>a</t>
         </is>
       </c>
       <c r="G198" t="inlineStr">
@@ -7902,7 +7902,7 @@
         </is>
       </c>
       <c r="B200" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="C200" t="inlineStr"/>
       <c r="D200" t="inlineStr">
@@ -7941,7 +7941,7 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>djaj</t>
+          <t>djej</t>
         </is>
       </c>
       <c r="B201" t="inlineStr"/>
@@ -7958,7 +7958,7 @@
       </c>
       <c r="F201" t="inlineStr">
         <is>
-          <t>a</t>
+          <t>e</t>
         </is>
       </c>
       <c r="G201" t="inlineStr">
@@ -8007,7 +8007,7 @@
         </is>
       </c>
       <c r="B203" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C203" t="inlineStr"/>
       <c r="D203" t="inlineStr">
@@ -8015,17 +8015,17 @@
           <t>د</t>
         </is>
       </c>
-      <c r="E203" t="inlineStr">
+      <c r="E203" t="inlineStr"/>
+      <c r="F203" t="inlineStr">
         <is>
           <t>ج</t>
         </is>
       </c>
-      <c r="F203" t="inlineStr">
+      <c r="G203" t="inlineStr">
         <is>
           <t>ا</t>
         </is>
       </c>
-      <c r="G203" t="inlineStr"/>
       <c r="H203" t="inlineStr">
         <is>
           <t>ج</t>
@@ -8046,7 +8046,7 @@
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>djeij</t>
+          <t>dajaj</t>
         </is>
       </c>
       <c r="B204" t="inlineStr"/>
@@ -8058,17 +8058,17 @@
       </c>
       <c r="E204" t="inlineStr">
         <is>
+          <t>a</t>
+        </is>
+      </c>
+      <c r="F204" t="inlineStr">
+        <is>
           <t>j</t>
         </is>
       </c>
-      <c r="F204" t="inlineStr">
-        <is>
-          <t>e</t>
-        </is>
-      </c>
       <c r="G204" t="inlineStr">
         <is>
-          <t>i</t>
+          <t>a</t>
         </is>
       </c>
       <c r="H204" t="inlineStr">
@@ -8116,7 +8116,7 @@
         </is>
       </c>
       <c r="B206" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C206" t="inlineStr"/>
       <c r="D206" t="inlineStr">
@@ -8124,17 +8124,17 @@
           <t>د</t>
         </is>
       </c>
-      <c r="E206" t="inlineStr"/>
+      <c r="E206" t="inlineStr">
+        <is>
+          <t>ج</t>
+        </is>
+      </c>
       <c r="F206" t="inlineStr">
         <is>
-          <t>ج</t>
-        </is>
-      </c>
-      <c r="G206" t="inlineStr">
-        <is>
           <t>ا</t>
         </is>
       </c>
+      <c r="G206" t="inlineStr"/>
       <c r="H206" t="inlineStr">
         <is>
           <t>ج</t>
@@ -8155,7 +8155,7 @@
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>dajaj</t>
+          <t>djeij</t>
         </is>
       </c>
       <c r="B207" t="inlineStr"/>
@@ -8167,17 +8167,17 @@
       </c>
       <c r="E207" t="inlineStr">
         <is>
-          <t>a</t>
+          <t>j</t>
         </is>
       </c>
       <c r="F207" t="inlineStr">
         <is>
-          <t>j</t>
+          <t>e</t>
         </is>
       </c>
       <c r="G207" t="inlineStr">
         <is>
-          <t>a</t>
+          <t>i</t>
         </is>
       </c>
       <c r="H207" t="inlineStr">
@@ -8406,11 +8406,27 @@
         <v>1</v>
       </c>
       <c r="C215" t="inlineStr"/>
-      <c r="D215" t="inlineStr"/>
+      <c r="D215" t="inlineStr">
+        <is>
+          <t>ج</t>
+        </is>
+      </c>
       <c r="E215" t="inlineStr"/>
-      <c r="F215" t="inlineStr"/>
-      <c r="G215" t="inlineStr"/>
-      <c r="H215" t="inlineStr"/>
+      <c r="F215" t="inlineStr">
+        <is>
+          <t>ر</t>
+        </is>
+      </c>
+      <c r="G215" t="inlineStr">
+        <is>
+          <t>ا</t>
+        </is>
+      </c>
+      <c r="H215" t="inlineStr">
+        <is>
+          <t>ج</t>
+        </is>
+      </c>
       <c r="I215" t="inlineStr"/>
       <c r="J215" t="inlineStr"/>
       <c r="K215" t="inlineStr"/>
@@ -8426,16 +8442,36 @@
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>jraj?</t>
+          <t>jaraj</t>
         </is>
       </c>
       <c r="B216" t="inlineStr"/>
       <c r="C216" t="inlineStr"/>
-      <c r="D216" t="inlineStr"/>
-      <c r="E216" t="inlineStr"/>
-      <c r="F216" t="inlineStr"/>
-      <c r="G216" t="inlineStr"/>
-      <c r="H216" t="inlineStr"/>
+      <c r="D216" t="inlineStr">
+        <is>
+          <t>j</t>
+        </is>
+      </c>
+      <c r="E216" t="inlineStr">
+        <is>
+          <t>a</t>
+        </is>
+      </c>
+      <c r="F216" t="inlineStr">
+        <is>
+          <t>r</t>
+        </is>
+      </c>
+      <c r="G216" t="inlineStr">
+        <is>
+          <t>a</t>
+        </is>
+      </c>
+      <c r="H216" t="inlineStr">
+        <is>
+          <t>j</t>
+        </is>
+      </c>
       <c r="I216" t="inlineStr"/>
       <c r="J216" t="inlineStr"/>
       <c r="K216" t="inlineStr"/>
@@ -8479,27 +8515,11 @@
         <v>1</v>
       </c>
       <c r="C218" t="inlineStr"/>
-      <c r="D218" t="inlineStr">
-        <is>
-          <t>ج</t>
-        </is>
-      </c>
+      <c r="D218" t="inlineStr"/>
       <c r="E218" t="inlineStr"/>
-      <c r="F218" t="inlineStr">
-        <is>
-          <t>ر</t>
-        </is>
-      </c>
-      <c r="G218" t="inlineStr">
-        <is>
-          <t>ا</t>
-        </is>
-      </c>
-      <c r="H218" t="inlineStr">
-        <is>
-          <t>ج</t>
-        </is>
-      </c>
+      <c r="F218" t="inlineStr"/>
+      <c r="G218" t="inlineStr"/>
+      <c r="H218" t="inlineStr"/>
       <c r="I218" t="inlineStr"/>
       <c r="J218" t="inlineStr"/>
       <c r="K218" t="inlineStr"/>
@@ -8515,36 +8535,16 @@
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>jaraj</t>
+          <t>jraj?</t>
         </is>
       </c>
       <c r="B219" t="inlineStr"/>
       <c r="C219" t="inlineStr"/>
-      <c r="D219" t="inlineStr">
-        <is>
-          <t>j</t>
-        </is>
-      </c>
-      <c r="E219" t="inlineStr">
-        <is>
-          <t>a</t>
-        </is>
-      </c>
-      <c r="F219" t="inlineStr">
-        <is>
-          <t>r</t>
-        </is>
-      </c>
-      <c r="G219" t="inlineStr">
-        <is>
-          <t>a</t>
-        </is>
-      </c>
-      <c r="H219" t="inlineStr">
-        <is>
-          <t>j</t>
-        </is>
-      </c>
+      <c r="D219" t="inlineStr"/>
+      <c r="E219" t="inlineStr"/>
+      <c r="F219" t="inlineStr"/>
+      <c r="G219" t="inlineStr"/>
+      <c r="H219" t="inlineStr"/>
       <c r="I219" t="inlineStr"/>
       <c r="J219" t="inlineStr"/>
       <c r="K219" t="inlineStr"/>
@@ -8585,30 +8585,14 @@
         </is>
       </c>
       <c r="B221" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="C221" t="inlineStr"/>
-      <c r="D221" t="inlineStr">
-        <is>
-          <t>ج</t>
-        </is>
-      </c>
+      <c r="D221" t="inlineStr"/>
       <c r="E221" t="inlineStr"/>
-      <c r="F221" t="inlineStr">
-        <is>
-          <t>ر</t>
-        </is>
-      </c>
-      <c r="G221" t="inlineStr">
-        <is>
-          <t>ا</t>
-        </is>
-      </c>
-      <c r="H221" t="inlineStr">
-        <is>
-          <t>ج</t>
-        </is>
-      </c>
+      <c r="F221" t="inlineStr"/>
+      <c r="G221" t="inlineStr"/>
+      <c r="H221" t="inlineStr"/>
       <c r="I221" t="inlineStr"/>
       <c r="J221" t="inlineStr"/>
       <c r="K221" t="inlineStr"/>
@@ -8624,41 +8608,17 @@
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>garage</t>
+          <t>jerrah</t>
         </is>
       </c>
       <c r="B222" t="inlineStr"/>
       <c r="C222" t="inlineStr"/>
-      <c r="D222" t="inlineStr">
-        <is>
-          <t>g</t>
-        </is>
-      </c>
-      <c r="E222" t="inlineStr">
-        <is>
-          <t>a</t>
-        </is>
-      </c>
-      <c r="F222" t="inlineStr">
-        <is>
-          <t>r</t>
-        </is>
-      </c>
-      <c r="G222" t="inlineStr">
-        <is>
-          <t>a</t>
-        </is>
-      </c>
-      <c r="H222" t="inlineStr">
-        <is>
-          <t>g</t>
-        </is>
-      </c>
-      <c r="I222" t="inlineStr">
-        <is>
-          <t>e</t>
-        </is>
-      </c>
+      <c r="D222" t="inlineStr"/>
+      <c r="E222" t="inlineStr"/>
+      <c r="F222" t="inlineStr"/>
+      <c r="G222" t="inlineStr"/>
+      <c r="H222" t="inlineStr"/>
+      <c r="I222" t="inlineStr"/>
       <c r="J222" t="inlineStr"/>
       <c r="K222" t="inlineStr"/>
       <c r="L222" t="inlineStr"/>
@@ -8721,7 +8681,7 @@
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
-          <t xml:space="preserve">jira7 </t>
+          <t>jarrah</t>
         </is>
       </c>
       <c r="B225" t="inlineStr"/>
@@ -8794,7 +8754,7 @@
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>jarrah</t>
+          <t xml:space="preserve">jira7 </t>
         </is>
       </c>
       <c r="B228" t="inlineStr"/>
@@ -8844,14 +8804,30 @@
         </is>
       </c>
       <c r="B230" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="C230" t="inlineStr"/>
-      <c r="D230" t="inlineStr"/>
+      <c r="D230" t="inlineStr">
+        <is>
+          <t>ج</t>
+        </is>
+      </c>
       <c r="E230" t="inlineStr"/>
-      <c r="F230" t="inlineStr"/>
-      <c r="G230" t="inlineStr"/>
-      <c r="H230" t="inlineStr"/>
+      <c r="F230" t="inlineStr">
+        <is>
+          <t>ر</t>
+        </is>
+      </c>
+      <c r="G230" t="inlineStr">
+        <is>
+          <t>ا</t>
+        </is>
+      </c>
+      <c r="H230" t="inlineStr">
+        <is>
+          <t>ج</t>
+        </is>
+      </c>
       <c r="I230" t="inlineStr"/>
       <c r="J230" t="inlineStr"/>
       <c r="K230" t="inlineStr"/>
@@ -8867,17 +8843,41 @@
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>jerrah</t>
+          <t>garage</t>
         </is>
       </c>
       <c r="B231" t="inlineStr"/>
       <c r="C231" t="inlineStr"/>
-      <c r="D231" t="inlineStr"/>
-      <c r="E231" t="inlineStr"/>
-      <c r="F231" t="inlineStr"/>
-      <c r="G231" t="inlineStr"/>
-      <c r="H231" t="inlineStr"/>
-      <c r="I231" t="inlineStr"/>
+      <c r="D231" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="E231" t="inlineStr">
+        <is>
+          <t>a</t>
+        </is>
+      </c>
+      <c r="F231" t="inlineStr">
+        <is>
+          <t>r</t>
+        </is>
+      </c>
+      <c r="G231" t="inlineStr">
+        <is>
+          <t>a</t>
+        </is>
+      </c>
+      <c r="H231" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="I231" t="inlineStr">
+        <is>
+          <t>e</t>
+        </is>
+      </c>
       <c r="J231" t="inlineStr"/>
       <c r="K231" t="inlineStr"/>
       <c r="L231" t="inlineStr"/>
@@ -9462,14 +9462,14 @@
     <row r="252">
       <c r="A252" t="inlineStr">
         <is>
-          <t>haje</t>
+          <t>7aje</t>
         </is>
       </c>
       <c r="B252" t="inlineStr"/>
       <c r="C252" t="inlineStr"/>
       <c r="D252" t="inlineStr">
         <is>
-          <t>h</t>
+          <t>7</t>
         </is>
       </c>
       <c r="E252" t="inlineStr">
@@ -9563,14 +9563,14 @@
     <row r="255">
       <c r="A255" t="inlineStr">
         <is>
-          <t>7aje</t>
+          <t>haje</t>
         </is>
       </c>
       <c r="B255" t="inlineStr"/>
       <c r="C255" t="inlineStr"/>
       <c r="D255" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>h</t>
         </is>
       </c>
       <c r="E255" t="inlineStr">
@@ -9629,7 +9629,7 @@
         </is>
       </c>
       <c r="B257" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="C257" t="inlineStr"/>
       <c r="D257" t="inlineStr">
@@ -9668,7 +9668,7 @@
     <row r="258">
       <c r="A258" t="inlineStr">
         <is>
-          <t>sabah</t>
+          <t>sebe7</t>
         </is>
       </c>
       <c r="B258" t="inlineStr"/>
@@ -9680,7 +9680,7 @@
       </c>
       <c r="E258" t="inlineStr">
         <is>
-          <t>a</t>
+          <t>e</t>
         </is>
       </c>
       <c r="F258" t="inlineStr">
@@ -9690,12 +9690,12 @@
       </c>
       <c r="G258" t="inlineStr">
         <is>
-          <t>a</t>
+          <t>e</t>
         </is>
       </c>
       <c r="H258" t="inlineStr">
         <is>
-          <t>h</t>
+          <t>7</t>
         </is>
       </c>
       <c r="I258" t="inlineStr"/>
@@ -9738,7 +9738,7 @@
         </is>
       </c>
       <c r="B260" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="C260" t="inlineStr"/>
       <c r="D260" t="inlineStr">
@@ -9777,7 +9777,7 @@
     <row r="261">
       <c r="A261" t="inlineStr">
         <is>
-          <t>sebe7</t>
+          <t>saba7</t>
         </is>
       </c>
       <c r="B261" t="inlineStr"/>
@@ -9789,7 +9789,7 @@
       </c>
       <c r="E261" t="inlineStr">
         <is>
-          <t>e</t>
+          <t>a</t>
         </is>
       </c>
       <c r="F261" t="inlineStr">
@@ -9799,7 +9799,7 @@
       </c>
       <c r="G261" t="inlineStr">
         <is>
-          <t>e</t>
+          <t>a</t>
         </is>
       </c>
       <c r="H261" t="inlineStr">
@@ -9847,7 +9847,7 @@
         </is>
       </c>
       <c r="B263" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C263" t="inlineStr"/>
       <c r="D263" t="inlineStr">
@@ -9886,7 +9886,7 @@
     <row r="264">
       <c r="A264" t="inlineStr">
         <is>
-          <t>saba7</t>
+          <t>sabah</t>
         </is>
       </c>
       <c r="B264" t="inlineStr"/>
@@ -9913,7 +9913,7 @@
       </c>
       <c r="H264" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>h</t>
         </is>
       </c>
       <c r="I264" t="inlineStr"/>
@@ -9956,7 +9956,7 @@
         </is>
       </c>
       <c r="B266" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="C266" t="inlineStr"/>
       <c r="D266" t="inlineStr">
@@ -9995,7 +9995,7 @@
     <row r="267">
       <c r="A267" t="inlineStr">
         <is>
-          <t>5amsi</t>
+          <t>5amse</t>
         </is>
       </c>
       <c r="B267" t="inlineStr"/>
@@ -10022,7 +10022,7 @@
       </c>
       <c r="H267" t="inlineStr">
         <is>
-          <t>i</t>
+          <t>e</t>
         </is>
       </c>
       <c r="I267" t="inlineStr"/>
@@ -10065,7 +10065,7 @@
         </is>
       </c>
       <c r="B269" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="C269" t="inlineStr"/>
       <c r="D269" t="inlineStr">
@@ -10104,7 +10104,7 @@
     <row r="270">
       <c r="A270" t="inlineStr">
         <is>
-          <t>5amse</t>
+          <t>5amsi</t>
         </is>
       </c>
       <c r="B270" t="inlineStr"/>
@@ -10131,7 +10131,7 @@
       </c>
       <c r="H270" t="inlineStr">
         <is>
-          <t>e</t>
+          <t>i</t>
         </is>
       </c>
       <c r="I270" t="inlineStr"/>
@@ -10174,7 +10174,7 @@
         </is>
       </c>
       <c r="B272" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="C272" t="inlineStr"/>
       <c r="D272" t="inlineStr">
@@ -10213,7 +10213,7 @@
     <row r="273">
       <c r="A273" t="inlineStr">
         <is>
-          <t>khamsa</t>
+          <t>khamse</t>
         </is>
       </c>
       <c r="B273" t="inlineStr"/>
@@ -10240,7 +10240,7 @@
       </c>
       <c r="H273" t="inlineStr">
         <is>
-          <t>a</t>
+          <t>e</t>
         </is>
       </c>
       <c r="I273" t="inlineStr"/>
@@ -10283,7 +10283,7 @@
         </is>
       </c>
       <c r="B275" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="C275" t="inlineStr"/>
       <c r="D275" t="inlineStr">
@@ -10322,7 +10322,7 @@
     <row r="276">
       <c r="A276" t="inlineStr">
         <is>
-          <t>khamse</t>
+          <t>khamsa</t>
         </is>
       </c>
       <c r="B276" t="inlineStr"/>
@@ -10349,7 +10349,7 @@
       </c>
       <c r="H276" t="inlineStr">
         <is>
-          <t>e</t>
+          <t>a</t>
         </is>
       </c>
       <c r="I276" t="inlineStr"/>
@@ -10750,14 +10750,14 @@
     <row r="288">
       <c r="A288" t="inlineStr">
         <is>
-          <t>chawerma</t>
+          <t>shawerma</t>
         </is>
       </c>
       <c r="B288" t="inlineStr"/>
       <c r="C288" t="inlineStr"/>
       <c r="D288" t="inlineStr">
         <is>
-          <t>ch</t>
+          <t>sh</t>
         </is>
       </c>
       <c r="E288" t="inlineStr">
@@ -11000,14 +11000,14 @@
     <row r="294">
       <c r="A294" t="inlineStr">
         <is>
-          <t>shawerma</t>
+          <t>chawarma</t>
         </is>
       </c>
       <c r="B294" t="inlineStr"/>
       <c r="C294" t="inlineStr"/>
       <c r="D294" t="inlineStr">
         <is>
-          <t>sh</t>
+          <t>ch</t>
         </is>
       </c>
       <c r="E294" t="inlineStr">
@@ -11022,7 +11022,7 @@
       </c>
       <c r="G294" t="inlineStr">
         <is>
-          <t>e</t>
+          <t>a</t>
         </is>
       </c>
       <c r="H294" t="inlineStr">
@@ -11125,7 +11125,7 @@
     <row r="297">
       <c r="A297" t="inlineStr">
         <is>
-          <t>chawarma</t>
+          <t>chawerma</t>
         </is>
       </c>
       <c r="B297" t="inlineStr"/>
@@ -11147,7 +11147,7 @@
       </c>
       <c r="G297" t="inlineStr">
         <is>
-          <t>a</t>
+          <t>e</t>
         </is>
       </c>
       <c r="H297" t="inlineStr">
@@ -11437,7 +11437,7 @@
         </is>
       </c>
       <c r="B305" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C305" t="inlineStr"/>
       <c r="D305" t="inlineStr">
@@ -11480,7 +11480,7 @@
     <row r="306">
       <c r="A306" t="inlineStr">
         <is>
-          <t>sahtein</t>
+          <t>sa7tein</t>
         </is>
       </c>
       <c r="B306" t="inlineStr"/>
@@ -11497,7 +11497,7 @@
       </c>
       <c r="F306" t="inlineStr">
         <is>
-          <t>h</t>
+          <t>7</t>
         </is>
       </c>
       <c r="G306" t="inlineStr">
@@ -11554,7 +11554,7 @@
         </is>
       </c>
       <c r="B308" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C308" t="inlineStr"/>
       <c r="D308" t="inlineStr">
@@ -11597,7 +11597,7 @@
     <row r="309">
       <c r="A309" t="inlineStr">
         <is>
-          <t>sa7tein</t>
+          <t>sahtein</t>
         </is>
       </c>
       <c r="B309" t="inlineStr"/>
@@ -11614,7 +11614,7 @@
       </c>
       <c r="F309" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>h</t>
         </is>
       </c>
       <c r="G309" t="inlineStr">
@@ -11909,15 +11909,31 @@
         </is>
       </c>
       <c r="B317" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="C317" t="inlineStr"/>
-      <c r="D317" t="inlineStr"/>
+      <c r="D317" t="inlineStr">
+        <is>
+          <t>م</t>
+        </is>
+      </c>
       <c r="E317" t="inlineStr"/>
-      <c r="F317" t="inlineStr"/>
-      <c r="G317" t="inlineStr"/>
+      <c r="F317" t="inlineStr">
+        <is>
+          <t>ض</t>
+        </is>
+      </c>
+      <c r="G317" t="inlineStr">
+        <is>
+          <t>ط</t>
+        </is>
+      </c>
       <c r="H317" t="inlineStr"/>
-      <c r="I317" t="inlineStr"/>
+      <c r="I317" t="inlineStr">
+        <is>
+          <t>ر</t>
+        </is>
+      </c>
       <c r="J317" t="inlineStr"/>
       <c r="K317" t="inlineStr"/>
       <c r="L317" t="inlineStr"/>
@@ -11932,17 +11948,41 @@
     <row r="318">
       <c r="A318" t="inlineStr">
         <is>
-          <t>mitdar</t>
+          <t>medtar</t>
         </is>
       </c>
       <c r="B318" t="inlineStr"/>
       <c r="C318" t="inlineStr"/>
-      <c r="D318" t="inlineStr"/>
-      <c r="E318" t="inlineStr"/>
-      <c r="F318" t="inlineStr"/>
-      <c r="G318" t="inlineStr"/>
-      <c r="H318" t="inlineStr"/>
-      <c r="I318" t="inlineStr"/>
+      <c r="D318" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="E318" t="inlineStr">
+        <is>
+          <t>e</t>
+        </is>
+      </c>
+      <c r="F318" t="inlineStr">
+        <is>
+          <t>d</t>
+        </is>
+      </c>
+      <c r="G318" t="inlineStr">
+        <is>
+          <t>t</t>
+        </is>
+      </c>
+      <c r="H318" t="inlineStr">
+        <is>
+          <t>a</t>
+        </is>
+      </c>
+      <c r="I318" t="inlineStr">
+        <is>
+          <t>r</t>
+        </is>
+      </c>
       <c r="J318" t="inlineStr"/>
       <c r="K318" t="inlineStr"/>
       <c r="L318" t="inlineStr"/>
@@ -11982,31 +12022,15 @@
         </is>
       </c>
       <c r="B320" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C320" t="inlineStr"/>
-      <c r="D320" t="inlineStr">
-        <is>
-          <t>م</t>
-        </is>
-      </c>
+      <c r="D320" t="inlineStr"/>
       <c r="E320" t="inlineStr"/>
-      <c r="F320" t="inlineStr">
-        <is>
-          <t>ض</t>
-        </is>
-      </c>
-      <c r="G320" t="inlineStr">
-        <is>
-          <t>ط</t>
-        </is>
-      </c>
+      <c r="F320" t="inlineStr"/>
+      <c r="G320" t="inlineStr"/>
       <c r="H320" t="inlineStr"/>
-      <c r="I320" t="inlineStr">
-        <is>
-          <t>ر</t>
-        </is>
-      </c>
+      <c r="I320" t="inlineStr"/>
       <c r="J320" t="inlineStr"/>
       <c r="K320" t="inlineStr"/>
       <c r="L320" t="inlineStr"/>
@@ -12021,41 +12045,17 @@
     <row r="321">
       <c r="A321" t="inlineStr">
         <is>
-          <t>mettar</t>
+          <t>mitdar</t>
         </is>
       </c>
       <c r="B321" t="inlineStr"/>
       <c r="C321" t="inlineStr"/>
-      <c r="D321" t="inlineStr">
-        <is>
-          <t>m</t>
-        </is>
-      </c>
-      <c r="E321" t="inlineStr">
-        <is>
-          <t>e</t>
-        </is>
-      </c>
-      <c r="F321" t="inlineStr">
-        <is>
-          <t>t</t>
-        </is>
-      </c>
-      <c r="G321" t="inlineStr">
-        <is>
-          <t>t</t>
-        </is>
-      </c>
-      <c r="H321" t="inlineStr">
-        <is>
-          <t>a</t>
-        </is>
-      </c>
-      <c r="I321" t="inlineStr">
-        <is>
-          <t>r</t>
-        </is>
-      </c>
+      <c r="D321" t="inlineStr"/>
+      <c r="E321" t="inlineStr"/>
+      <c r="F321" t="inlineStr"/>
+      <c r="G321" t="inlineStr"/>
+      <c r="H321" t="inlineStr"/>
+      <c r="I321" t="inlineStr"/>
       <c r="J321" t="inlineStr"/>
       <c r="K321" t="inlineStr"/>
       <c r="L321" t="inlineStr"/>
@@ -12095,7 +12095,7 @@
         </is>
       </c>
       <c r="B323" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C323" t="inlineStr"/>
       <c r="D323" t="inlineStr">
@@ -12134,7 +12134,7 @@
     <row r="324">
       <c r="A324" t="inlineStr">
         <is>
-          <t>modtar</t>
+          <t>mettar</t>
         </is>
       </c>
       <c r="B324" t="inlineStr"/>
@@ -12146,12 +12146,12 @@
       </c>
       <c r="E324" t="inlineStr">
         <is>
-          <t>o</t>
+          <t>e</t>
         </is>
       </c>
       <c r="F324" t="inlineStr">
         <is>
-          <t>d</t>
+          <t>t</t>
         </is>
       </c>
       <c r="G324" t="inlineStr">
@@ -12208,7 +12208,7 @@
         </is>
       </c>
       <c r="B326" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="C326" t="inlineStr"/>
       <c r="D326" t="inlineStr">
@@ -12247,7 +12247,7 @@
     <row r="327">
       <c r="A327" t="inlineStr">
         <is>
-          <t>medtar</t>
+          <t>modtar</t>
         </is>
       </c>
       <c r="B327" t="inlineStr"/>
@@ -12259,7 +12259,7 @@
       </c>
       <c r="E327" t="inlineStr">
         <is>
-          <t>e</t>
+          <t>o</t>
         </is>
       </c>
       <c r="F327" t="inlineStr">
@@ -12321,7 +12321,7 @@
         </is>
       </c>
       <c r="B329" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="C329" t="inlineStr"/>
       <c r="D329" t="inlineStr">
@@ -12364,7 +12364,7 @@
     <row r="330">
       <c r="A330" t="inlineStr">
         <is>
-          <t>tawla</t>
+          <t>tewla</t>
         </is>
       </c>
       <c r="B330" t="inlineStr"/>
@@ -12376,7 +12376,7 @@
       </c>
       <c r="E330" t="inlineStr">
         <is>
-          <t>a</t>
+          <t>e</t>
         </is>
       </c>
       <c r="F330" t="inlineStr">
@@ -12434,7 +12434,7 @@
         </is>
       </c>
       <c r="B332" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="C332" t="inlineStr"/>
       <c r="D332" t="inlineStr">
@@ -12477,7 +12477,7 @@
     <row r="333">
       <c r="A333" t="inlineStr">
         <is>
-          <t>tewla</t>
+          <t>tawle</t>
         </is>
       </c>
       <c r="B333" t="inlineStr"/>
@@ -12489,22 +12489,22 @@
       </c>
       <c r="E333" t="inlineStr">
         <is>
+          <t>a</t>
+        </is>
+      </c>
+      <c r="F333" t="inlineStr">
+        <is>
+          <t>w</t>
+        </is>
+      </c>
+      <c r="G333" t="inlineStr">
+        <is>
+          <t>l</t>
+        </is>
+      </c>
+      <c r="H333" t="inlineStr">
+        <is>
           <t>e</t>
-        </is>
-      </c>
-      <c r="F333" t="inlineStr">
-        <is>
-          <t>w</t>
-        </is>
-      </c>
-      <c r="G333" t="inlineStr">
-        <is>
-          <t>l</t>
-        </is>
-      </c>
-      <c r="H333" t="inlineStr">
-        <is>
-          <t>a</t>
         </is>
       </c>
       <c r="I333" t="inlineStr"/>
@@ -12547,7 +12547,7 @@
         </is>
       </c>
       <c r="B335" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C335" t="inlineStr"/>
       <c r="D335" t="inlineStr">
@@ -12590,7 +12590,7 @@
     <row r="336">
       <c r="A336" t="inlineStr">
         <is>
-          <t>tawle</t>
+          <t>tawla</t>
         </is>
       </c>
       <c r="B336" t="inlineStr"/>
@@ -12617,7 +12617,7 @@
       </c>
       <c r="H336" t="inlineStr">
         <is>
-          <t>e</t>
+          <t>a</t>
         </is>
       </c>
       <c r="I336" t="inlineStr"/>
@@ -12820,7 +12820,7 @@
     <row r="342">
       <c r="A342" t="inlineStr">
         <is>
-          <t>muzahara</t>
+          <t>mozahara</t>
         </is>
       </c>
       <c r="B342" t="inlineStr"/>
@@ -12832,7 +12832,7 @@
       </c>
       <c r="E342" t="inlineStr">
         <is>
-          <t>u</t>
+          <t>o</t>
         </is>
       </c>
       <c r="F342" t="inlineStr">
@@ -12949,7 +12949,7 @@
     <row r="345">
       <c r="A345" t="inlineStr">
         <is>
-          <t>mozahara</t>
+          <t>muzahara</t>
         </is>
       </c>
       <c r="B345" t="inlineStr"/>
@@ -12961,7 +12961,7 @@
       </c>
       <c r="E345" t="inlineStr">
         <is>
-          <t>o</t>
+          <t>u</t>
         </is>
       </c>
       <c r="F345" t="inlineStr">
@@ -13273,7 +13273,7 @@
         </is>
       </c>
       <c r="B353" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="C353" t="inlineStr"/>
       <c r="D353" t="inlineStr">
@@ -13312,14 +13312,14 @@
     <row r="354">
       <c r="A354" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 8arib</t>
+          <t>gharib</t>
         </is>
       </c>
       <c r="B354" t="inlineStr"/>
       <c r="C354" t="inlineStr"/>
       <c r="D354" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>gh</t>
         </is>
       </c>
       <c r="E354" t="inlineStr">
@@ -13382,7 +13382,7 @@
         </is>
       </c>
       <c r="B356" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="C356" t="inlineStr"/>
       <c r="D356" t="inlineStr">
@@ -13421,14 +13421,14 @@
     <row r="357">
       <c r="A357" t="inlineStr">
         <is>
-          <t>gharib</t>
+          <t xml:space="preserve"> 8arib</t>
         </is>
       </c>
       <c r="B357" t="inlineStr"/>
       <c r="C357" t="inlineStr"/>
       <c r="D357" t="inlineStr">
         <is>
-          <t>gh</t>
+          <t>8</t>
         </is>
       </c>
       <c r="E357" t="inlineStr">
@@ -13530,7 +13530,7 @@
     <row r="360">
       <c r="A360" t="inlineStr">
         <is>
-          <t>ghareeb</t>
+          <t xml:space="preserve">gharib </t>
         </is>
       </c>
       <c r="B360" t="inlineStr"/>
@@ -13552,7 +13552,7 @@
       </c>
       <c r="G360" t="inlineStr">
         <is>
-          <t>ee</t>
+          <t>i</t>
         </is>
       </c>
       <c r="H360" t="inlineStr">
@@ -13639,7 +13639,7 @@
     <row r="363">
       <c r="A363" t="inlineStr">
         <is>
-          <t xml:space="preserve">gharib </t>
+          <t>ghareeb</t>
         </is>
       </c>
       <c r="B363" t="inlineStr"/>
@@ -13661,7 +13661,7 @@
       </c>
       <c r="G363" t="inlineStr">
         <is>
-          <t>i</t>
+          <t>ee</t>
         </is>
       </c>
       <c r="H363" t="inlineStr">
@@ -13709,7 +13709,7 @@
         </is>
       </c>
       <c r="B365" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C365" t="inlineStr"/>
       <c r="D365" t="inlineStr">
@@ -13752,7 +13752,7 @@
     <row r="366">
       <c r="A366" t="inlineStr">
         <is>
-          <t>falefil</t>
+          <t>falefel</t>
         </is>
       </c>
       <c r="B366" t="inlineStr"/>
@@ -13784,7 +13784,7 @@
       </c>
       <c r="I366" t="inlineStr">
         <is>
-          <t>i</t>
+          <t>e</t>
         </is>
       </c>
       <c r="J366" t="inlineStr">
@@ -13830,7 +13830,7 @@
         </is>
       </c>
       <c r="B368" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="C368" t="inlineStr"/>
       <c r="D368" t="inlineStr">
@@ -13873,7 +13873,7 @@
     <row r="369">
       <c r="A369" t="inlineStr">
         <is>
-          <t>falefel</t>
+          <t>falafel</t>
         </is>
       </c>
       <c r="B369" t="inlineStr"/>
@@ -13895,7 +13895,7 @@
       </c>
       <c r="G369" t="inlineStr">
         <is>
-          <t>e</t>
+          <t>a</t>
         </is>
       </c>
       <c r="H369" t="inlineStr">
@@ -13951,7 +13951,7 @@
         </is>
       </c>
       <c r="B371" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="C371" t="inlineStr"/>
       <c r="D371" t="inlineStr">
@@ -13994,7 +13994,7 @@
     <row r="372">
       <c r="A372" t="inlineStr">
         <is>
-          <t>falafel</t>
+          <t>falefil</t>
         </is>
       </c>
       <c r="B372" t="inlineStr"/>
@@ -14016,7 +14016,7 @@
       </c>
       <c r="G372" t="inlineStr">
         <is>
-          <t>a</t>
+          <t>e</t>
         </is>
       </c>
       <c r="H372" t="inlineStr">
@@ -14026,7 +14026,7 @@
       </c>
       <c r="I372" t="inlineStr">
         <is>
-          <t>e</t>
+          <t>i</t>
         </is>
       </c>
       <c r="J372" t="inlineStr">
@@ -14111,7 +14111,7 @@
     <row r="375">
       <c r="A375" t="inlineStr">
         <is>
-          <t>r2e2</t>
+          <t>rkik</t>
         </is>
       </c>
       <c r="B375" t="inlineStr"/>
@@ -14123,17 +14123,17 @@
       </c>
       <c r="E375" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>k</t>
         </is>
       </c>
       <c r="F375" t="inlineStr">
         <is>
-          <t>e</t>
+          <t>i</t>
         </is>
       </c>
       <c r="G375" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>k</t>
         </is>
       </c>
       <c r="H375" t="inlineStr"/>
@@ -14321,7 +14321,7 @@
     <row r="381">
       <c r="A381" t="inlineStr">
         <is>
-          <t>rkik</t>
+          <t>r2e2</t>
         </is>
       </c>
       <c r="B381" t="inlineStr"/>
@@ -14333,17 +14333,17 @@
       </c>
       <c r="E381" t="inlineStr">
         <is>
-          <t>k</t>
+          <t>2</t>
         </is>
       </c>
       <c r="F381" t="inlineStr">
         <is>
-          <t>i</t>
+          <t>e</t>
         </is>
       </c>
       <c r="G381" t="inlineStr">
         <is>
-          <t>k</t>
+          <t>2</t>
         </is>
       </c>
       <c r="H381" t="inlineStr"/>
@@ -15356,7 +15356,7 @@
         </is>
       </c>
       <c r="B410" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="C410" t="inlineStr"/>
       <c r="D410" t="inlineStr">
@@ -15395,7 +15395,7 @@
     <row r="411">
       <c r="A411" t="inlineStr">
         <is>
-          <t>shamaa</t>
+          <t>sham3a</t>
         </is>
       </c>
       <c r="B411" t="inlineStr"/>
@@ -15417,7 +15417,7 @@
       </c>
       <c r="G411" t="inlineStr">
         <is>
-          <t>a</t>
+          <t>3</t>
         </is>
       </c>
       <c r="H411" t="inlineStr">
@@ -15465,7 +15465,7 @@
         </is>
       </c>
       <c r="B413" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="C413" t="inlineStr"/>
       <c r="D413" t="inlineStr">
@@ -15504,7 +15504,7 @@
     <row r="414">
       <c r="A414" t="inlineStr">
         <is>
-          <t>cham3a</t>
+          <t>chamaa</t>
         </is>
       </c>
       <c r="B414" t="inlineStr"/>
@@ -15526,7 +15526,7 @@
       </c>
       <c r="G414" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>a</t>
         </is>
       </c>
       <c r="H414" t="inlineStr">
@@ -15574,7 +15574,7 @@
         </is>
       </c>
       <c r="B416" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C416" t="inlineStr"/>
       <c r="D416" t="inlineStr">
@@ -15613,14 +15613,14 @@
     <row r="417">
       <c r="A417" t="inlineStr">
         <is>
-          <t>chamaa</t>
+          <t>shamaa</t>
         </is>
       </c>
       <c r="B417" t="inlineStr"/>
       <c r="C417" t="inlineStr"/>
       <c r="D417" t="inlineStr">
         <is>
-          <t>ch</t>
+          <t>sh</t>
         </is>
       </c>
       <c r="E417" t="inlineStr">
@@ -15722,14 +15722,14 @@
     <row r="420">
       <c r="A420" t="inlineStr">
         <is>
-          <t>sham3a</t>
+          <t>cham3a</t>
         </is>
       </c>
       <c r="B420" t="inlineStr"/>
       <c r="C420" t="inlineStr"/>
       <c r="D420" t="inlineStr">
         <is>
-          <t>sh</t>
+          <t>ch</t>
         </is>
       </c>
       <c r="E420" t="inlineStr">
@@ -15815,7 +15815,7 @@
     <row r="423">
       <c r="A423" t="inlineStr">
         <is>
-          <t>hadika</t>
+          <t>7adi2a</t>
         </is>
       </c>
       <c r="B423" t="inlineStr"/>
@@ -15961,7 +15961,7 @@
     <row r="429">
       <c r="A429" t="inlineStr">
         <is>
-          <t>7adi2a</t>
+          <t>hadika</t>
         </is>
       </c>
       <c r="B429" t="inlineStr"/>
@@ -16042,7 +16042,7 @@
       </c>
       <c r="J431" t="inlineStr">
         <is>
-          <t> </t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="K431" t="inlineStr">
@@ -16115,7 +16115,7 @@
       </c>
       <c r="J432" t="inlineStr">
         <is>
-          <t> </t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="K432" t="inlineStr"/>
@@ -16207,7 +16207,7 @@
       </c>
       <c r="J434" t="inlineStr">
         <is>
-          <t> </t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="K434" t="inlineStr">
@@ -16225,12 +16225,12 @@
           <t>و</t>
         </is>
       </c>
-      <c r="N434" t="inlineStr"/>
-      <c r="O434" t="inlineStr">
+      <c r="N434" t="inlineStr">
         <is>
           <t>ر</t>
         </is>
       </c>
+      <c r="O434" t="inlineStr"/>
       <c r="P434" t="inlineStr"/>
       <c r="Q434" t="inlineStr">
         <is>
@@ -16243,14 +16243,14 @@
     <row r="435">
       <c r="A435" t="inlineStr">
         <is>
-          <t>7adi2et wared</t>
+          <t>hadi2et wroud</t>
         </is>
       </c>
       <c r="B435" t="inlineStr"/>
       <c r="C435" t="inlineStr"/>
       <c r="D435" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>h</t>
         </is>
       </c>
       <c r="E435" t="inlineStr">
@@ -16280,7 +16280,7 @@
       </c>
       <c r="J435" t="inlineStr">
         <is>
-          <t> </t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="K435" t="inlineStr"/>
@@ -16292,17 +16292,17 @@
       </c>
       <c r="N435" t="inlineStr">
         <is>
-          <t>a</t>
+          <t>r</t>
         </is>
       </c>
       <c r="O435" t="inlineStr">
         <is>
-          <t>r</t>
+          <t>o</t>
         </is>
       </c>
       <c r="P435" t="inlineStr">
         <is>
-          <t>e</t>
+          <t>u</t>
         </is>
       </c>
       <c r="Q435" t="inlineStr">
@@ -16372,7 +16372,7 @@
       </c>
       <c r="J437" t="inlineStr">
         <is>
-          <t> </t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="K437" t="inlineStr">
@@ -16390,12 +16390,12 @@
           <t>و</t>
         </is>
       </c>
-      <c r="N437" t="inlineStr">
+      <c r="N437" t="inlineStr"/>
+      <c r="O437" t="inlineStr">
         <is>
           <t>ر</t>
         </is>
       </c>
-      <c r="O437" t="inlineStr"/>
       <c r="P437" t="inlineStr"/>
       <c r="Q437" t="inlineStr">
         <is>
@@ -16408,14 +16408,14 @@
     <row r="438">
       <c r="A438" t="inlineStr">
         <is>
-          <t>hadi2et wroud</t>
+          <t>7adi2et wared</t>
         </is>
       </c>
       <c r="B438" t="inlineStr"/>
       <c r="C438" t="inlineStr"/>
       <c r="D438" t="inlineStr">
         <is>
-          <t>h</t>
+          <t>7</t>
         </is>
       </c>
       <c r="E438" t="inlineStr">
@@ -16445,7 +16445,7 @@
       </c>
       <c r="J438" t="inlineStr">
         <is>
-          <t> </t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="K438" t="inlineStr"/>
@@ -16457,17 +16457,17 @@
       </c>
       <c r="N438" t="inlineStr">
         <is>
+          <t>a</t>
+        </is>
+      </c>
+      <c r="O438" t="inlineStr">
+        <is>
           <t>r</t>
         </is>
       </c>
-      <c r="O438" t="inlineStr">
-        <is>
-          <t>o</t>
-        </is>
-      </c>
       <c r="P438" t="inlineStr">
         <is>
-          <t>u</t>
+          <t>e</t>
         </is>
       </c>
       <c r="Q438" t="inlineStr">
@@ -16537,7 +16537,7 @@
       </c>
       <c r="J440" t="inlineStr">
         <is>
-          <t> </t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="K440" t="inlineStr">
@@ -16610,7 +16610,7 @@
       </c>
       <c r="J441" t="inlineStr">
         <is>
-          <t> </t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="K441" t="inlineStr"/>
@@ -16621,7 +16621,7 @@
       </c>
       <c r="M441" t="inlineStr">
         <is>
-          <t> </t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="N441" t="inlineStr">
@@ -16706,7 +16706,7 @@
       </c>
       <c r="J443" t="inlineStr">
         <is>
-          <t> </t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="K443" t="inlineStr">
@@ -16779,7 +16779,7 @@
       </c>
       <c r="J444" t="inlineStr">
         <is>
-          <t> </t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="K444" t="inlineStr">
@@ -16868,57 +16868,57 @@
           <t>ق</t>
         </is>
       </c>
-      <c r="I446" t="inlineStr">
+      <c r="I446" t="inlineStr"/>
+      <c r="J446" t="inlineStr">
         <is>
           <t>ة</t>
         </is>
       </c>
-      <c r="J446" t="inlineStr">
-        <is>
-          <t> </t>
-        </is>
-      </c>
       <c r="K446" t="inlineStr">
         <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="L446" t="inlineStr">
+        <is>
           <t>ا</t>
         </is>
       </c>
-      <c r="L446" t="inlineStr">
+      <c r="M446" t="inlineStr">
         <is>
           <t>ل</t>
         </is>
       </c>
-      <c r="M446" t="inlineStr"/>
-      <c r="N446" t="inlineStr">
+      <c r="N446" t="inlineStr"/>
+      <c r="O446" t="inlineStr">
         <is>
           <t>و</t>
         </is>
       </c>
-      <c r="O446" t="inlineStr"/>
-      <c r="P446" t="inlineStr">
+      <c r="P446" t="inlineStr"/>
+      <c r="Q446" t="inlineStr">
         <is>
           <t>ر</t>
         </is>
       </c>
-      <c r="Q446" t="inlineStr">
+      <c r="R446" t="inlineStr"/>
+      <c r="S446" t="inlineStr">
         <is>
           <t>د</t>
         </is>
       </c>
-      <c r="R446" t="inlineStr"/>
-      <c r="S446" t="inlineStr"/>
     </row>
     <row r="447">
       <c r="A447" t="inlineStr">
         <is>
-          <t>7adi2et el ward</t>
+          <t>hadi2it l wared</t>
         </is>
       </c>
       <c r="B447" t="inlineStr"/>
       <c r="C447" t="inlineStr"/>
       <c r="D447" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>h</t>
         </is>
       </c>
       <c r="E447" t="inlineStr">
@@ -16943,51 +16943,55 @@
       </c>
       <c r="I447" t="inlineStr">
         <is>
-          <t>et</t>
+          <t>i</t>
         </is>
       </c>
       <c r="J447" t="inlineStr">
         <is>
-          <t> </t>
+          <t>t</t>
         </is>
       </c>
       <c r="K447" t="inlineStr">
         <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="L447" t="inlineStr"/>
+      <c r="M447" t="inlineStr">
+        <is>
+          <t>l</t>
+        </is>
+      </c>
+      <c r="N447" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="O447" t="inlineStr">
+        <is>
+          <t>w</t>
+        </is>
+      </c>
+      <c r="P447" t="inlineStr">
+        <is>
+          <t>a</t>
+        </is>
+      </c>
+      <c r="Q447" t="inlineStr">
+        <is>
+          <t>r</t>
+        </is>
+      </c>
+      <c r="R447" t="inlineStr">
+        <is>
           <t>e</t>
         </is>
       </c>
-      <c r="L447" t="inlineStr">
-        <is>
-          <t>l</t>
-        </is>
-      </c>
-      <c r="M447" t="inlineStr">
-        <is>
-          <t> </t>
-        </is>
-      </c>
-      <c r="N447" t="inlineStr">
-        <is>
-          <t>w</t>
-        </is>
-      </c>
-      <c r="O447" t="inlineStr">
-        <is>
-          <t>a</t>
-        </is>
-      </c>
-      <c r="P447" t="inlineStr">
-        <is>
-          <t>r</t>
-        </is>
-      </c>
-      <c r="Q447" t="inlineStr">
+      <c r="S447" t="inlineStr">
         <is>
           <t>d</t>
         </is>
       </c>
-      <c r="R447" t="inlineStr"/>
-      <c r="S447" t="inlineStr"/>
     </row>
     <row r="448">
       <c r="A448" t="inlineStr"/>
@@ -17020,150 +17024,46 @@
         <v>1</v>
       </c>
       <c r="C449" t="inlineStr"/>
-      <c r="D449" t="inlineStr">
-        <is>
-          <t>ح</t>
-        </is>
-      </c>
+      <c r="D449" t="inlineStr"/>
       <c r="E449" t="inlineStr"/>
-      <c r="F449" t="inlineStr">
-        <is>
-          <t>د</t>
-        </is>
-      </c>
-      <c r="G449" t="inlineStr">
-        <is>
-          <t>ي</t>
-        </is>
-      </c>
-      <c r="H449" t="inlineStr">
-        <is>
-          <t>ق</t>
-        </is>
-      </c>
+      <c r="F449" t="inlineStr"/>
+      <c r="G449" t="inlineStr"/>
+      <c r="H449" t="inlineStr"/>
       <c r="I449" t="inlineStr"/>
-      <c r="J449" t="inlineStr">
-        <is>
-          <t>ة</t>
-        </is>
-      </c>
-      <c r="K449" t="inlineStr">
-        <is>
-          <t> </t>
-        </is>
-      </c>
-      <c r="L449" t="inlineStr">
-        <is>
-          <t>ا</t>
-        </is>
-      </c>
-      <c r="M449" t="inlineStr">
-        <is>
-          <t>ل</t>
-        </is>
-      </c>
+      <c r="J449" t="inlineStr"/>
+      <c r="K449" t="inlineStr"/>
+      <c r="L449" t="inlineStr"/>
+      <c r="M449" t="inlineStr"/>
       <c r="N449" t="inlineStr"/>
-      <c r="O449" t="inlineStr">
-        <is>
-          <t>و</t>
-        </is>
-      </c>
+      <c r="O449" t="inlineStr"/>
       <c r="P449" t="inlineStr"/>
-      <c r="Q449" t="inlineStr">
-        <is>
-          <t>ر</t>
-        </is>
-      </c>
-      <c r="R449" t="inlineStr">
-        <is>
-          <t>د</t>
-        </is>
-      </c>
+      <c r="Q449" t="inlineStr"/>
+      <c r="R449" t="inlineStr"/>
       <c r="S449" t="inlineStr"/>
     </row>
     <row r="450">
       <c r="A450" t="inlineStr">
         <is>
-          <t>hadi2it el ward</t>
+          <t>jnaynet l wared</t>
         </is>
       </c>
       <c r="B450" t="inlineStr"/>
       <c r="C450" t="inlineStr"/>
-      <c r="D450" t="inlineStr">
-        <is>
-          <t>h</t>
-        </is>
-      </c>
-      <c r="E450" t="inlineStr">
-        <is>
-          <t>a</t>
-        </is>
-      </c>
-      <c r="F450" t="inlineStr">
-        <is>
-          <t>d</t>
-        </is>
-      </c>
-      <c r="G450" t="inlineStr">
-        <is>
-          <t>i</t>
-        </is>
-      </c>
-      <c r="H450" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="I450" t="inlineStr">
-        <is>
-          <t>i</t>
-        </is>
-      </c>
-      <c r="J450" t="inlineStr">
-        <is>
-          <t>t</t>
-        </is>
-      </c>
-      <c r="K450" t="inlineStr">
-        <is>
-          <t> </t>
-        </is>
-      </c>
-      <c r="L450" t="inlineStr">
-        <is>
-          <t>e</t>
-        </is>
-      </c>
-      <c r="M450" t="inlineStr">
-        <is>
-          <t>l</t>
-        </is>
-      </c>
-      <c r="N450" t="inlineStr">
-        <is>
-          <t> </t>
-        </is>
-      </c>
-      <c r="O450" t="inlineStr">
-        <is>
-          <t>w</t>
-        </is>
-      </c>
-      <c r="P450" t="inlineStr">
-        <is>
-          <t>a</t>
-        </is>
-      </c>
-      <c r="Q450" t="inlineStr">
-        <is>
-          <t>r</t>
-        </is>
-      </c>
-      <c r="R450" t="inlineStr">
-        <is>
-          <t>d</t>
-        </is>
-      </c>
+      <c r="D450" t="inlineStr"/>
+      <c r="E450" t="inlineStr"/>
+      <c r="F450" t="inlineStr"/>
+      <c r="G450" t="inlineStr"/>
+      <c r="H450" t="inlineStr"/>
+      <c r="I450" t="inlineStr"/>
+      <c r="J450" t="inlineStr"/>
+      <c r="K450" t="inlineStr"/>
+      <c r="L450" t="inlineStr"/>
+      <c r="M450" t="inlineStr"/>
+      <c r="N450" t="inlineStr"/>
+      <c r="O450" t="inlineStr"/>
+      <c r="P450" t="inlineStr"/>
+      <c r="Q450" t="inlineStr"/>
+      <c r="R450" t="inlineStr"/>
       <c r="S450" t="inlineStr"/>
     </row>
     <row r="451">
@@ -17197,46 +17097,150 @@
         <v>1</v>
       </c>
       <c r="C452" t="inlineStr"/>
-      <c r="D452" t="inlineStr"/>
+      <c r="D452" t="inlineStr">
+        <is>
+          <t>ح</t>
+        </is>
+      </c>
       <c r="E452" t="inlineStr"/>
-      <c r="F452" t="inlineStr"/>
-      <c r="G452" t="inlineStr"/>
-      <c r="H452" t="inlineStr"/>
+      <c r="F452" t="inlineStr">
+        <is>
+          <t>د</t>
+        </is>
+      </c>
+      <c r="G452" t="inlineStr">
+        <is>
+          <t>ي</t>
+        </is>
+      </c>
+      <c r="H452" t="inlineStr">
+        <is>
+          <t>ق</t>
+        </is>
+      </c>
       <c r="I452" t="inlineStr"/>
-      <c r="J452" t="inlineStr"/>
-      <c r="K452" t="inlineStr"/>
-      <c r="L452" t="inlineStr"/>
-      <c r="M452" t="inlineStr"/>
+      <c r="J452" t="inlineStr">
+        <is>
+          <t>ة</t>
+        </is>
+      </c>
+      <c r="K452" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="L452" t="inlineStr">
+        <is>
+          <t>ا</t>
+        </is>
+      </c>
+      <c r="M452" t="inlineStr">
+        <is>
+          <t>ل</t>
+        </is>
+      </c>
       <c r="N452" t="inlineStr"/>
-      <c r="O452" t="inlineStr"/>
+      <c r="O452" t="inlineStr">
+        <is>
+          <t>و</t>
+        </is>
+      </c>
       <c r="P452" t="inlineStr"/>
-      <c r="Q452" t="inlineStr"/>
-      <c r="R452" t="inlineStr"/>
+      <c r="Q452" t="inlineStr">
+        <is>
+          <t>ر</t>
+        </is>
+      </c>
+      <c r="R452" t="inlineStr">
+        <is>
+          <t>د</t>
+        </is>
+      </c>
       <c r="S452" t="inlineStr"/>
     </row>
     <row r="453">
       <c r="A453" t="inlineStr">
         <is>
-          <t>jnaynet l wared</t>
+          <t>hadi2it el ward</t>
         </is>
       </c>
       <c r="B453" t="inlineStr"/>
       <c r="C453" t="inlineStr"/>
-      <c r="D453" t="inlineStr"/>
-      <c r="E453" t="inlineStr"/>
-      <c r="F453" t="inlineStr"/>
-      <c r="G453" t="inlineStr"/>
-      <c r="H453" t="inlineStr"/>
-      <c r="I453" t="inlineStr"/>
-      <c r="J453" t="inlineStr"/>
-      <c r="K453" t="inlineStr"/>
-      <c r="L453" t="inlineStr"/>
-      <c r="M453" t="inlineStr"/>
-      <c r="N453" t="inlineStr"/>
-      <c r="O453" t="inlineStr"/>
-      <c r="P453" t="inlineStr"/>
-      <c r="Q453" t="inlineStr"/>
-      <c r="R453" t="inlineStr"/>
+      <c r="D453" t="inlineStr">
+        <is>
+          <t>h</t>
+        </is>
+      </c>
+      <c r="E453" t="inlineStr">
+        <is>
+          <t>a</t>
+        </is>
+      </c>
+      <c r="F453" t="inlineStr">
+        <is>
+          <t>d</t>
+        </is>
+      </c>
+      <c r="G453" t="inlineStr">
+        <is>
+          <t>i</t>
+        </is>
+      </c>
+      <c r="H453" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I453" t="inlineStr">
+        <is>
+          <t>i</t>
+        </is>
+      </c>
+      <c r="J453" t="inlineStr">
+        <is>
+          <t>t</t>
+        </is>
+      </c>
+      <c r="K453" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="L453" t="inlineStr">
+        <is>
+          <t>e</t>
+        </is>
+      </c>
+      <c r="M453" t="inlineStr">
+        <is>
+          <t>l</t>
+        </is>
+      </c>
+      <c r="N453" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="O453" t="inlineStr">
+        <is>
+          <t>w</t>
+        </is>
+      </c>
+      <c r="P453" t="inlineStr">
+        <is>
+          <t>a</t>
+        </is>
+      </c>
+      <c r="Q453" t="inlineStr">
+        <is>
+          <t>r</t>
+        </is>
+      </c>
+      <c r="R453" t="inlineStr">
+        <is>
+          <t>d</t>
+        </is>
+      </c>
       <c r="S453" t="inlineStr"/>
     </row>
     <row r="454">
@@ -17291,57 +17295,57 @@
           <t>ق</t>
         </is>
       </c>
-      <c r="I455" t="inlineStr"/>
+      <c r="I455" t="inlineStr">
+        <is>
+          <t>ة</t>
+        </is>
+      </c>
       <c r="J455" t="inlineStr">
         <is>
-          <t>ة</t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="K455" t="inlineStr">
         <is>
-          <t> </t>
+          <t>ا</t>
         </is>
       </c>
       <c r="L455" t="inlineStr">
         <is>
-          <t>ا</t>
-        </is>
-      </c>
-      <c r="M455" t="inlineStr">
-        <is>
           <t>ل</t>
         </is>
       </c>
-      <c r="N455" t="inlineStr"/>
-      <c r="O455" t="inlineStr">
+      <c r="M455" t="inlineStr"/>
+      <c r="N455" t="inlineStr">
         <is>
           <t>و</t>
         </is>
       </c>
-      <c r="P455" t="inlineStr"/>
+      <c r="O455" t="inlineStr"/>
+      <c r="P455" t="inlineStr">
+        <is>
+          <t>ر</t>
+        </is>
+      </c>
       <c r="Q455" t="inlineStr">
         <is>
-          <t>ر</t>
+          <t>د</t>
         </is>
       </c>
       <c r="R455" t="inlineStr"/>
-      <c r="S455" t="inlineStr">
-        <is>
-          <t>د</t>
-        </is>
-      </c>
+      <c r="S455" t="inlineStr"/>
     </row>
     <row r="456">
       <c r="A456" t="inlineStr">
         <is>
-          <t>hadi2it l wared</t>
+          <t>7adi2et el ward</t>
         </is>
       </c>
       <c r="B456" t="inlineStr"/>
       <c r="C456" t="inlineStr"/>
       <c r="D456" t="inlineStr">
         <is>
-          <t>h</t>
+          <t>7</t>
         </is>
       </c>
       <c r="E456" t="inlineStr">
@@ -17366,55 +17370,51 @@
       </c>
       <c r="I456" t="inlineStr">
         <is>
-          <t>i</t>
+          <t>et</t>
         </is>
       </c>
       <c r="J456" t="inlineStr">
         <is>
-          <t>t</t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="K456" t="inlineStr">
         <is>
-          <t> </t>
-        </is>
-      </c>
-      <c r="L456" t="inlineStr"/>
+          <t>e</t>
+        </is>
+      </c>
+      <c r="L456" t="inlineStr">
+        <is>
+          <t>l</t>
+        </is>
+      </c>
       <c r="M456" t="inlineStr">
         <is>
-          <t>l</t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="N456" t="inlineStr">
         <is>
-          <t> </t>
+          <t>w</t>
         </is>
       </c>
       <c r="O456" t="inlineStr">
         <is>
-          <t>w</t>
+          <t>a</t>
         </is>
       </c>
       <c r="P456" t="inlineStr">
         <is>
-          <t>a</t>
+          <t>r</t>
         </is>
       </c>
       <c r="Q456" t="inlineStr">
         <is>
-          <t>r</t>
-        </is>
-      </c>
-      <c r="R456" t="inlineStr">
-        <is>
-          <t>e</t>
-        </is>
-      </c>
-      <c r="S456" t="inlineStr">
-        <is>
           <t>d</t>
         </is>
       </c>
+      <c r="R456" t="inlineStr"/>
+      <c r="S456" t="inlineStr"/>
     </row>
     <row r="457">
       <c r="A457" t="inlineStr"/>
@@ -17475,7 +17475,7 @@
       </c>
       <c r="J458" t="inlineStr">
         <is>
-          <t> </t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="K458" t="inlineStr">
@@ -17548,7 +17548,7 @@
       </c>
       <c r="J459" t="inlineStr">
         <is>
-          <t> </t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="K459" t="inlineStr">
@@ -17563,7 +17563,7 @@
       </c>
       <c r="M459" t="inlineStr">
         <is>
-          <t> </t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="N459" t="inlineStr">
@@ -17653,7 +17653,7 @@
       </c>
       <c r="K461" t="inlineStr">
         <is>
-          <t> </t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="L461" t="inlineStr">
@@ -17730,7 +17730,7 @@
       </c>
       <c r="K462" t="inlineStr">
         <is>
-          <t> </t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="L462" t="inlineStr">
@@ -17745,7 +17745,7 @@
       </c>
       <c r="N462" t="inlineStr">
         <is>
-          <t> </t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="O462" t="inlineStr">
@@ -18262,7 +18262,7 @@
         </is>
       </c>
       <c r="B476" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C476" t="inlineStr"/>
       <c r="D476" t="inlineStr">
@@ -18301,7 +18301,7 @@
     <row r="477">
       <c r="A477" t="inlineStr">
         <is>
-          <t>wahde</t>
+          <t>wa7di</t>
         </is>
       </c>
       <c r="B477" t="inlineStr"/>
@@ -18318,7 +18318,7 @@
       </c>
       <c r="F477" t="inlineStr">
         <is>
-          <t>h</t>
+          <t>7</t>
         </is>
       </c>
       <c r="G477" t="inlineStr">
@@ -18328,7 +18328,7 @@
       </c>
       <c r="H477" t="inlineStr">
         <is>
-          <t>e</t>
+          <t>i</t>
         </is>
       </c>
       <c r="I477" t="inlineStr"/>
@@ -18371,7 +18371,7 @@
         </is>
       </c>
       <c r="B479" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C479" t="inlineStr"/>
       <c r="D479" t="inlineStr">
@@ -18410,7 +18410,7 @@
     <row r="480">
       <c r="A480" t="inlineStr">
         <is>
-          <t>wa7di</t>
+          <t>wa7de</t>
         </is>
       </c>
       <c r="B480" t="inlineStr"/>
@@ -18437,7 +18437,7 @@
       </c>
       <c r="H480" t="inlineStr">
         <is>
-          <t>i</t>
+          <t>e</t>
         </is>
       </c>
       <c r="I480" t="inlineStr"/>
@@ -18519,7 +18519,7 @@
     <row r="483">
       <c r="A483" t="inlineStr">
         <is>
-          <t>wa7de</t>
+          <t>wahde</t>
         </is>
       </c>
       <c r="B483" t="inlineStr"/>
@@ -18536,7 +18536,7 @@
       </c>
       <c r="F483" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>h</t>
         </is>
       </c>
       <c r="G483" t="inlineStr">
@@ -18662,7 +18662,7 @@
         </is>
       </c>
       <c r="B488" t="n">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="C488" t="inlineStr"/>
       <c r="D488" t="inlineStr">
@@ -18670,12 +18670,12 @@
           <t>م</t>
         </is>
       </c>
-      <c r="E488" t="inlineStr"/>
-      <c r="F488" t="inlineStr">
+      <c r="E488" t="inlineStr">
         <is>
           <t>ع</t>
         </is>
       </c>
+      <c r="F488" t="inlineStr"/>
       <c r="G488" t="inlineStr">
         <is>
           <t>ر</t>
@@ -18705,7 +18705,7 @@
     <row r="489">
       <c r="A489" t="inlineStr">
         <is>
-          <t>ma3rouf</t>
+          <t>maarouf</t>
         </is>
       </c>
       <c r="B489" t="inlineStr"/>
@@ -18722,7 +18722,7 @@
       </c>
       <c r="F489" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>a</t>
         </is>
       </c>
       <c r="G489" t="inlineStr">
@@ -18779,7 +18779,7 @@
         </is>
       </c>
       <c r="B491" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="C491" t="inlineStr"/>
       <c r="D491" t="inlineStr">
@@ -18787,12 +18787,12 @@
           <t>م</t>
         </is>
       </c>
-      <c r="E491" t="inlineStr">
+      <c r="E491" t="inlineStr"/>
+      <c r="F491" t="inlineStr">
         <is>
           <t>ع</t>
         </is>
       </c>
-      <c r="F491" t="inlineStr"/>
       <c r="G491" t="inlineStr">
         <is>
           <t>ر</t>
@@ -18822,7 +18822,7 @@
     <row r="492">
       <c r="A492" t="inlineStr">
         <is>
-          <t>maarouf</t>
+          <t>ma3rouf</t>
         </is>
       </c>
       <c r="B492" t="inlineStr"/>
@@ -18839,7 +18839,7 @@
       </c>
       <c r="F492" t="inlineStr">
         <is>
-          <t>a</t>
+          <t>3</t>
         </is>
       </c>
       <c r="G492" t="inlineStr">
@@ -19171,7 +19171,7 @@
         </is>
       </c>
       <c r="B503" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C503" t="inlineStr"/>
       <c r="D503" t="inlineStr">
@@ -19206,14 +19206,14 @@
     <row r="504">
       <c r="A504" t="inlineStr">
         <is>
-          <t>helo</t>
+          <t>7elo</t>
         </is>
       </c>
       <c r="B504" t="inlineStr"/>
       <c r="C504" t="inlineStr"/>
       <c r="D504" t="inlineStr">
         <is>
-          <t>h</t>
+          <t>7</t>
         </is>
       </c>
       <c r="E504" t="inlineStr">
@@ -19272,7 +19272,7 @@
         </is>
       </c>
       <c r="B506" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C506" t="inlineStr"/>
       <c r="D506" t="inlineStr">
@@ -19307,19 +19307,19 @@
     <row r="507">
       <c r="A507" t="inlineStr">
         <is>
-          <t>7elo</t>
+          <t>hilu</t>
         </is>
       </c>
       <c r="B507" t="inlineStr"/>
       <c r="C507" t="inlineStr"/>
       <c r="D507" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>h</t>
         </is>
       </c>
       <c r="E507" t="inlineStr">
         <is>
-          <t>e</t>
+          <t>i</t>
         </is>
       </c>
       <c r="F507" t="inlineStr">
@@ -19329,7 +19329,7 @@
       </c>
       <c r="G507" t="inlineStr">
         <is>
-          <t>o</t>
+          <t>u</t>
         </is>
       </c>
       <c r="H507" t="inlineStr"/>
@@ -19373,7 +19373,7 @@
         </is>
       </c>
       <c r="B509" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="C509" t="inlineStr"/>
       <c r="D509" t="inlineStr">
@@ -19408,7 +19408,7 @@
     <row r="510">
       <c r="A510" t="inlineStr">
         <is>
-          <t>hilu</t>
+          <t>helo</t>
         </is>
       </c>
       <c r="B510" t="inlineStr"/>
@@ -19420,7 +19420,7 @@
       </c>
       <c r="E510" t="inlineStr">
         <is>
-          <t>i</t>
+          <t>e</t>
         </is>
       </c>
       <c r="F510" t="inlineStr">
@@ -19430,7 +19430,7 @@
       </c>
       <c r="G510" t="inlineStr">
         <is>
-          <t>u</t>
+          <t>o</t>
         </is>
       </c>
       <c r="H510" t="inlineStr"/>
@@ -19575,7 +19575,7 @@
         </is>
       </c>
       <c r="B515" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="C515" t="inlineStr"/>
       <c r="D515" t="inlineStr">
@@ -19622,7 +19622,7 @@
     <row r="516">
       <c r="A516" t="inlineStr">
         <is>
-          <t>yasmin</t>
+          <t>yesmin</t>
         </is>
       </c>
       <c r="B516" t="inlineStr"/>
@@ -19634,7 +19634,7 @@
       </c>
       <c r="E516" t="inlineStr">
         <is>
-          <t>a</t>
+          <t>e</t>
         </is>
       </c>
       <c r="F516" t="inlineStr">
@@ -19696,7 +19696,7 @@
         </is>
       </c>
       <c r="B518" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="C518" t="inlineStr"/>
       <c r="D518" t="inlineStr">
@@ -19743,7 +19743,7 @@
     <row r="519">
       <c r="A519" t="inlineStr">
         <is>
-          <t>yesmin</t>
+          <t>yasmin</t>
         </is>
       </c>
       <c r="B519" t="inlineStr"/>
@@ -19755,7 +19755,7 @@
       </c>
       <c r="E519" t="inlineStr">
         <is>
-          <t>e</t>
+          <t>a</t>
         </is>
       </c>
       <c r="F519" t="inlineStr">

</xml_diff>